<commit_message>
dpm install && make format && make rm vol=logs
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -458,11 +458,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>34</v>
+        <v>500</v>
       </c>
     </row>
     <row r="3">
@@ -481,11 +481,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>73</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -504,11 +504,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5">
@@ -550,11 +550,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2733</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -573,11 +573,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>14</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8">
@@ -596,11 +596,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>78</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -619,11 +619,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>500</v>
+        <v>2733</v>
       </c>
     </row>
     <row r="10">
@@ -642,11 +642,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>395</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -660,16 +660,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>830</v>
       </c>
     </row>
     <row r="12">
@@ -688,11 +688,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>565</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -706,16 +706,16 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>830</v>
+        <v>395</v>
       </c>
     </row>
     <row r="14">
@@ -734,11 +734,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>565</v>
       </c>
     </row>
     <row r="15">
@@ -757,11 +757,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -803,11 +803,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>9150</v>
       </c>
     </row>
     <row r="18">
@@ -826,11 +826,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>3652</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="19">
@@ -867,16 +867,16 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>6352</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -895,11 +895,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>9150</v>
+        <v>3652</v>
       </c>
     </row>
     <row r="22">
@@ -913,16 +913,16 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1037</v>
+        <v>6352</v>
       </c>
     </row>
     <row r="23">
@@ -941,11 +941,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1259</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="24">
@@ -964,11 +964,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25">
@@ -987,11 +987,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26">
@@ -1005,16 +1005,16 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -1028,16 +1028,16 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28">
@@ -1056,11 +1056,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>38</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29">
@@ -1079,11 +1079,11 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -1097,16 +1097,16 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>85</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31">
@@ -1120,16 +1120,16 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>17</v>
+        <v>85</v>
       </c>
     </row>
     <row r="32">
@@ -1148,11 +1148,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33">
@@ -1166,16 +1166,16 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -1189,16 +1189,16 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
     </row>
     <row r="35">
@@ -1217,11 +1217,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>25</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36">
@@ -1281,16 +1281,16 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>223</v>
+        <v>468</v>
       </c>
     </row>
     <row r="39">
@@ -1327,16 +1327,16 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>468</v>
+        <v>223</v>
       </c>
     </row>
     <row r="41">
@@ -1355,11 +1355,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="42">
@@ -1378,11 +1378,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>432</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="43">
@@ -1419,16 +1419,16 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>761</v>
+        <v>432</v>
       </c>
     </row>
     <row r="45">
@@ -1447,11 +1447,11 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>1260</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
@@ -1465,16 +1465,16 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>1092</v>
+        <v>761</v>
       </c>
     </row>
     <row r="47">
@@ -1493,11 +1493,11 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>1335</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="48">
@@ -1516,11 +1516,11 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="49">
@@ -1539,11 +1539,11 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>22</v>
+        <v>39</v>
       </c>
     </row>
     <row r="50">
@@ -1585,11 +1585,11 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -1631,11 +1631,11 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="54">
@@ -1649,16 +1649,16 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>4</v>
+        <v>4428</v>
       </c>
     </row>
     <row r="55">
@@ -1677,11 +1677,11 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>750</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="56">
@@ -1695,16 +1695,16 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>4428</v>
+        <v>629</v>
       </c>
     </row>
     <row r="57">
@@ -1723,11 +1723,11 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>629</v>
+        <v>750</v>
       </c>
     </row>
     <row r="58">
@@ -1746,11 +1746,11 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>1213</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>7</v>
+        <v>109</v>
       </c>
     </row>
     <row r="60">
@@ -1787,16 +1787,16 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>430</v>
+        <v>78</v>
       </c>
     </row>
     <row r="61">
@@ -1810,16 +1810,16 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>109</v>
+        <v>430</v>
       </c>
     </row>
     <row r="62">
@@ -1838,11 +1838,11 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>78</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>119</v>
+        <v>42</v>
       </c>
     </row>
     <row r="65">
@@ -1902,16 +1902,16 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>524</v>
+        <v>41</v>
       </c>
     </row>
     <row r="66">
@@ -1930,11 +1930,11 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>41</v>
+        <v>119</v>
       </c>
     </row>
     <row r="67">
@@ -1948,16 +1948,16 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>42</v>
+        <v>524</v>
       </c>
     </row>
     <row r="68">
@@ -1976,11 +1976,11 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>3</v>
+        <v>2334</v>
       </c>
     </row>
     <row r="69">
@@ -1999,11 +1999,11 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>260</v>
+        <v>1598</v>
       </c>
     </row>
     <row r="70">
@@ -2022,11 +2022,11 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>3507</v>
       </c>
     </row>
     <row r="71">
@@ -2045,11 +2045,11 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>216</v>
+        <v>34063</v>
       </c>
     </row>
     <row r="72">
@@ -2068,11 +2068,11 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>37636</v>
+        <v>886</v>
       </c>
     </row>
     <row r="73">
@@ -2086,16 +2086,16 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>1598</v>
+        <v>37636</v>
       </c>
     </row>
     <row r="74">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>3507</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75">
@@ -2137,11 +2137,11 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>34063</v>
+        <v>260</v>
       </c>
     </row>
     <row r="76">
@@ -2155,16 +2155,16 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>886</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>2334</v>
+        <v>216</v>
       </c>
     </row>
     <row r="78">
@@ -2206,11 +2206,11 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>6</v>
+        <v>162087</v>
       </c>
     </row>
     <row r="79">
@@ -2229,11 +2229,11 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>4338</v>
+        <v>39786</v>
       </c>
     </row>
     <row r="80">
@@ -2247,16 +2247,16 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>22985</v>
+        <v>176905</v>
       </c>
     </row>
     <row r="81">
@@ -2270,16 +2270,16 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>176905</v>
+        <v>15695</v>
       </c>
     </row>
     <row r="82">
@@ -2298,11 +2298,11 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>162087</v>
+        <v>4338</v>
       </c>
     </row>
     <row r="83">
@@ -2321,11 +2321,11 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>39786</v>
+        <v>22985</v>
       </c>
     </row>
     <row r="84">
@@ -2344,11 +2344,11 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>15695</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85">
@@ -2367,11 +2367,11 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>4</v>
+        <v>84</v>
       </c>
     </row>
     <row r="86">
@@ -2390,11 +2390,11 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>159</v>
+        <v>3</v>
       </c>
     </row>
     <row r="87">
@@ -2408,16 +2408,16 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>285</v>
+        <v>7</v>
       </c>
     </row>
     <row r="88">
@@ -2436,11 +2436,11 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>84</v>
+        <v>4</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>3</v>
+        <v>159</v>
       </c>
     </row>
     <row r="90">
@@ -2477,16 +2477,16 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>7</v>
+        <v>285</v>
       </c>
     </row>
     <row r="91">
@@ -2505,11 +2505,11 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>8</v>
+        <v>200</v>
       </c>
     </row>
     <row r="92">
@@ -2528,11 +2528,11 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>55</v>
+        <v>112</v>
       </c>
     </row>
     <row r="93">
@@ -2546,16 +2546,16 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>83</v>
+        <v>55</v>
       </c>
     </row>
     <row r="94">
@@ -2574,11 +2574,11 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>112</v>
+        <v>8</v>
       </c>
     </row>
     <row r="95">
@@ -2592,16 +2592,16 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>200</v>
+        <v>83</v>
       </c>
     </row>
     <row r="96">
@@ -2620,11 +2620,11 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>7</v>
+        <v>516</v>
       </c>
     </row>
     <row r="97">
@@ -2638,16 +2638,16 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
     </row>
     <row r="98">
@@ -2661,16 +2661,16 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>13</v>
+        <v>123</v>
       </c>
     </row>
     <row r="99">
@@ -2689,11 +2689,11 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>516</v>
+        <v>88</v>
       </c>
     </row>
     <row r="100">
@@ -2712,11 +2712,11 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>123</v>
+        <v>7</v>
       </c>
     </row>
     <row r="101">
@@ -2735,11 +2735,11 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>2</v>
+        <v>705</v>
       </c>
     </row>
     <row r="102">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>22</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="103">
@@ -2776,16 +2776,16 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E103" t="n">
-        <v>3052</v>
+        <v>22</v>
       </c>
     </row>
     <row r="104">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>5200</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105">
@@ -2822,16 +2822,16 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>705</v>
+        <v>3052</v>
       </c>
     </row>
     <row r="106">
@@ -2850,11 +2850,11 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="107">
@@ -2868,16 +2868,16 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>87</v>
+        <v>397</v>
       </c>
     </row>
     <row r="108">
@@ -2891,16 +2891,16 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>397</v>
+        <v>81</v>
       </c>
     </row>
     <row r="109">
@@ -2919,11 +2919,11 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="110">
@@ -2942,11 +2942,11 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>6</v>
+        <v>974</v>
       </c>
     </row>
     <row r="111">
@@ -2965,11 +2965,11 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>974</v>
+        <v>4</v>
       </c>
     </row>
     <row r="112">
@@ -2988,11 +2988,11 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>7</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="113">
@@ -3011,11 +3011,11 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>1356</v>
+        <v>817</v>
       </c>
     </row>
     <row r="114">
@@ -3029,16 +3029,16 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>3</v>
+        <v>755</v>
       </c>
     </row>
     <row r="115">
@@ -3052,16 +3052,16 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>755</v>
+        <v>14404</v>
       </c>
     </row>
     <row r="116">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>1014</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="117">
@@ -3103,11 +3103,11 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>817</v>
+        <v>3</v>
       </c>
     </row>
     <row r="118">
@@ -3126,11 +3126,11 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>14404</v>
+        <v>7</v>
       </c>
     </row>
     <row r="119">
@@ -3149,11 +3149,11 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="120">
@@ -3172,11 +3172,11 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>337</v>
+        <v>189</v>
       </c>
     </row>
     <row r="121">
@@ -3190,16 +3190,16 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>135</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="122">
@@ -3213,16 +3213,16 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>1208</v>
+        <v>172</v>
       </c>
     </row>
     <row r="123">
@@ -3241,11 +3241,11 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>3</v>
+        <v>337</v>
       </c>
     </row>
     <row r="124">
@@ -3264,11 +3264,11 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>189</v>
+        <v>135</v>
       </c>
     </row>
     <row r="125">
@@ -3287,11 +3287,11 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>172</v>
+        <v>2</v>
       </c>
     </row>
     <row r="126">
@@ -3310,11 +3310,11 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E126" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E127" t="n">
-        <v>250</v>
+        <v>7</v>
       </c>
     </row>
     <row r="128">
@@ -3379,11 +3379,11 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="130">
@@ -3402,11 +3402,11 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>7</v>
+        <v>250</v>
       </c>
     </row>
     <row r="131">
@@ -3466,16 +3466,16 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E133" t="n">
-        <v>1584</v>
+        <v>701</v>
       </c>
     </row>
     <row r="134">
@@ -3489,16 +3489,16 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>701</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="135">
@@ -3517,11 +3517,11 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E135" t="n">
-        <v>10389</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="136">
@@ -3563,11 +3563,11 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E137" t="n">
-        <v>1332</v>
+        <v>10389</v>
       </c>
     </row>
     <row r="138">
@@ -3581,16 +3581,16 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E138" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="139">
@@ -3604,16 +3604,16 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E139" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="140">
@@ -3701,11 +3701,11 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E143" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
     </row>
     <row r="144">
@@ -3719,16 +3719,16 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="145">
@@ -3747,11 +3747,11 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>13</v>
+        <v>54</v>
       </c>
     </row>
     <row r="146">
@@ -3765,16 +3765,16 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="147">
@@ -3793,11 +3793,11 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148">
@@ -3816,11 +3816,11 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>44</v>
+        <v>4</v>
       </c>
     </row>
     <row r="149">
@@ -3839,11 +3839,11 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="150">
@@ -3862,11 +3862,11 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E150" t="n">
-        <v>4</v>
+        <v>44</v>
       </c>
     </row>
     <row r="151">
@@ -3885,11 +3885,11 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="152">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E152" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="153">
@@ -3931,11 +3931,11 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="154">
@@ -3977,11 +3977,11 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>5</v>
+        <v>85</v>
       </c>
     </row>
     <row r="156">
@@ -4000,11 +4000,11 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E156" t="n">
-        <v>85</v>
+        <v>2</v>
       </c>
     </row>
     <row r="157">
@@ -4023,11 +4023,11 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="158">
@@ -4046,11 +4046,11 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>54</v>
+        <v>10</v>
       </c>
     </row>
     <row r="159">
@@ -4069,11 +4069,11 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E159" t="n">
-        <v>2</v>
+        <v>54</v>
       </c>
     </row>
     <row r="160">
@@ -4092,11 +4092,11 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E160" t="n">
-        <v>687</v>
+        <v>2</v>
       </c>
     </row>
     <row r="161">
@@ -4138,11 +4138,11 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>531</v>
+        <v>58</v>
       </c>
     </row>
     <row r="163">
@@ -4161,11 +4161,11 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>2</v>
+        <v>687</v>
       </c>
     </row>
     <row r="164">
@@ -4184,11 +4184,11 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>58</v>
+        <v>531</v>
       </c>
     </row>
     <row r="165">
@@ -4225,16 +4225,16 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>54</v>
+        <v>13</v>
       </c>
     </row>
     <row r="167">
@@ -4253,11 +4253,11 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E167" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="168">
@@ -4271,16 +4271,16 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>3</v>
+        <v>54</v>
       </c>
     </row>
     <row r="169">
@@ -4299,11 +4299,11 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="170">
@@ -4317,16 +4317,16 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>283</v>
+        <v>2</v>
       </c>
     </row>
     <row r="171">
@@ -4340,16 +4340,16 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E171" t="n">
-        <v>38</v>
+        <v>283</v>
       </c>
     </row>
     <row r="172">
@@ -4368,11 +4368,11 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
     </row>
     <row r="173">
@@ -4391,11 +4391,11 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>2</v>
+        <v>150</v>
       </c>
     </row>
     <row r="174">
@@ -4437,11 +4437,11 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>150</v>
+        <v>58</v>
       </c>
     </row>
     <row r="176">
@@ -4455,16 +4455,16 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E176" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="177">
@@ -4478,16 +4478,16 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E177" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="178">
@@ -4506,11 +4506,11 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
     </row>
     <row r="179">
@@ -4575,11 +4575,11 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>96</v>
+        <v>21</v>
       </c>
     </row>
     <row r="182">
@@ -4621,11 +4621,11 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
     </row>
     <row r="184">
@@ -4662,16 +4662,16 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E185" t="n">
-        <v>387</v>
+        <v>4</v>
       </c>
     </row>
     <row r="186">
@@ -4713,11 +4713,11 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>214</v>
+        <v>206</v>
       </c>
     </row>
     <row r="188">
@@ -4736,11 +4736,11 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>206</v>
+        <v>214</v>
       </c>
     </row>
     <row r="189">
@@ -4754,16 +4754,16 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>4</v>
+        <v>387</v>
       </c>
     </row>
     <row r="190">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
     </row>
     <row r="192">
@@ -4828,11 +4828,11 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>48</v>
+        <v>120</v>
       </c>
     </row>
     <row r="193">
@@ -4851,11 +4851,11 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
     </row>
     <row r="194">
@@ -4874,11 +4874,11 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="195">
@@ -4892,12 +4892,12 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E195" t="n">
@@ -4920,11 +4920,11 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="197">
@@ -4943,11 +4943,11 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="198">
@@ -4961,12 +4961,12 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -4989,11 +4989,11 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="200">
@@ -5012,11 +5012,11 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>101</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E202" t="n">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E203" t="n">
@@ -5122,16 +5122,16 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="206">
@@ -5150,11 +5150,11 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207">
@@ -5168,16 +5168,16 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="208">
@@ -5196,11 +5196,11 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="209">
@@ -5237,16 +5237,16 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>147</v>
+        <v>104</v>
       </c>
     </row>
     <row r="211">
@@ -5265,11 +5265,11 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>104</v>
+        <v>44</v>
       </c>
     </row>
     <row r="212">
@@ -5288,11 +5288,11 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
     </row>
     <row r="213">
@@ -5311,11 +5311,11 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>23</v>
+        <v>68</v>
       </c>
     </row>
     <row r="214">
@@ -5352,16 +5352,16 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E215" t="n">
-        <v>68</v>
+        <v>147</v>
       </c>
     </row>
     <row r="216">
@@ -5375,16 +5375,16 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E216" t="n">
-        <v>63</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217">
@@ -5403,11 +5403,11 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E217" t="n">
-        <v>21</v>
+        <v>43</v>
       </c>
     </row>
     <row r="218">
@@ -5444,16 +5444,16 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E219" t="n">
-        <v>3</v>
+        <v>63</v>
       </c>
     </row>
     <row r="220">
@@ -5472,11 +5472,11 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E220" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="221">
@@ -5495,11 +5495,11 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E221" t="n">
-        <v>43</v>
+        <v>3</v>
       </c>
     </row>
     <row r="222">
@@ -5518,11 +5518,11 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E222" t="n">
-        <v>25</v>
+        <v>83</v>
       </c>
     </row>
     <row r="223">
@@ -5541,11 +5541,11 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E223" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="224">
@@ -5564,11 +5564,11 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E224" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="225">
@@ -5587,11 +5587,11 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E225" t="n">
-        <v>83</v>
+        <v>25</v>
       </c>
     </row>
     <row r="226">
@@ -5909,11 +5909,11 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>165</v>
+        <v>250</v>
       </c>
     </row>
     <row r="240">
@@ -5932,11 +5932,11 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E240" t="n">
-        <v>250</v>
+        <v>165</v>
       </c>
     </row>
     <row r="241">
@@ -5955,11 +5955,11 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E241" t="n">
-        <v>199</v>
+        <v>1</v>
       </c>
     </row>
     <row r="242">
@@ -5978,11 +5978,11 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E242" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="243">
@@ -6001,11 +6001,11 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E243" t="n">
-        <v>20</v>
+        <v>199</v>
       </c>
     </row>
     <row r="244">
@@ -6019,16 +6019,16 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>1482</v>
+        <v>3963</v>
       </c>
     </row>
     <row r="245">
@@ -6047,11 +6047,11 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>944</v>
+        <v>3879</v>
       </c>
     </row>
     <row r="246">
@@ -6065,16 +6065,16 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E246" t="n">
-        <v>3963</v>
+        <v>944</v>
       </c>
     </row>
     <row r="247">
@@ -6093,11 +6093,11 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E247" t="n">
-        <v>2</v>
+        <v>4103</v>
       </c>
     </row>
     <row r="248">
@@ -6116,11 +6116,11 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E248" t="n">
-        <v>3879</v>
+        <v>2</v>
       </c>
     </row>
     <row r="249">
@@ -6162,11 +6162,11 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>4103</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="251">
@@ -6180,16 +6180,16 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="252">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="253">
@@ -6249,16 +6249,16 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="255">
@@ -6277,11 +6277,11 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>477</v>
+        <v>283</v>
       </c>
     </row>
     <row r="256">
@@ -6300,11 +6300,11 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>29</v>
+        <v>477</v>
       </c>
     </row>
     <row r="257">
@@ -6323,11 +6323,11 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>283</v>
+        <v>547</v>
       </c>
     </row>
     <row r="258">
@@ -6369,11 +6369,11 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>547</v>
+        <v>29</v>
       </c>
     </row>
     <row r="260">
@@ -6410,16 +6410,16 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>1072</v>
+        <v>423</v>
       </c>
     </row>
     <row r="262">
@@ -6433,16 +6433,16 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E262" t="n">
-        <v>423</v>
+        <v>854</v>
       </c>
     </row>
     <row r="263">
@@ -6484,11 +6484,11 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>854</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="265">
@@ -6553,11 +6553,11 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>93</v>
+        <v>468</v>
       </c>
     </row>
     <row r="268">
@@ -6576,11 +6576,11 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>468</v>
+        <v>93</v>
       </c>
     </row>
     <row r="269">
@@ -6599,11 +6599,11 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>434</v>
+        <v>343</v>
       </c>
     </row>
     <row r="270">
@@ -6622,11 +6622,11 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>256</v>
+        <v>434</v>
       </c>
     </row>
     <row r="271">
@@ -6663,16 +6663,16 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>202</v>
+        <v>256</v>
       </c>
     </row>
     <row r="273">
@@ -6686,16 +6686,16 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>343</v>
+        <v>202</v>
       </c>
     </row>
     <row r="274">
@@ -6709,16 +6709,16 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>4</v>
+        <v>149</v>
       </c>
     </row>
     <row r="275">
@@ -6732,16 +6732,16 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>149</v>
+        <v>115</v>
       </c>
     </row>
     <row r="276">
@@ -6760,11 +6760,11 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
     </row>
     <row r="277">
@@ -6783,11 +6783,11 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>115</v>
+        <v>4</v>
       </c>
     </row>
     <row r="278">
@@ -6806,11 +6806,11 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
     </row>
     <row r="279">
@@ -6824,16 +6824,16 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>60</v>
+        <v>317</v>
       </c>
     </row>
     <row r="280">
@@ -6852,11 +6852,11 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>25</v>
+        <v>143</v>
       </c>
     </row>
     <row r="281">
@@ -6875,11 +6875,11 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>143</v>
+        <v>25</v>
       </c>
     </row>
     <row r="282">
@@ -6898,11 +6898,11 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>7</v>
+        <v>60</v>
       </c>
     </row>
     <row r="283">
@@ -6921,11 +6921,11 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>1674</v>
+        <v>7</v>
       </c>
     </row>
     <row r="284">
@@ -6939,16 +6939,16 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>317</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="285">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E285" t="n">
@@ -7013,11 +7013,11 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="288">
@@ -7036,11 +7036,11 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="289">
@@ -7054,16 +7054,16 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>858</v>
+        <v>538</v>
       </c>
     </row>
     <row r="290">
@@ -7082,11 +7082,11 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>4</v>
+        <v>858</v>
       </c>
     </row>
     <row r="291">
@@ -7105,11 +7105,11 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>16</v>
+        <v>38</v>
       </c>
     </row>
     <row r="292">
@@ -7128,11 +7128,11 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>38</v>
+        <v>297</v>
       </c>
     </row>
     <row r="293">
@@ -7146,16 +7146,16 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>538</v>
+        <v>4</v>
       </c>
     </row>
     <row r="294">
@@ -7174,11 +7174,11 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>297</v>
+        <v>16</v>
       </c>
     </row>
     <row r="295">
@@ -7220,11 +7220,11 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>87</v>
+        <v>15</v>
       </c>
     </row>
     <row r="297">
@@ -7266,11 +7266,11 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>15</v>
+        <v>87</v>
       </c>
     </row>
     <row r="299">
@@ -7289,11 +7289,11 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
     </row>
     <row r="300">
@@ -7312,11 +7312,11 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="301">
@@ -7335,11 +7335,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
     </row>
     <row r="302">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="303">
@@ -7381,11 +7381,11 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>48</v>
+        <v>66</v>
       </c>
     </row>
     <row r="304">
@@ -7404,11 +7404,11 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
     </row>
     <row r="305">
@@ -7427,11 +7427,11 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>66</v>
+        <v>3</v>
       </c>
     </row>
     <row r="306">

</xml_diff>

<commit_message>
commit para checar alterações do v3, fontes
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -458,11 +458,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>34</v>
+        <v>500</v>
       </c>
     </row>
     <row r="3">
@@ -481,11 +481,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>73</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -504,11 +504,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5">
@@ -550,11 +550,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2733</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -573,11 +573,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>14</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8">
@@ -596,11 +596,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>78</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -619,11 +619,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>500</v>
+        <v>2733</v>
       </c>
     </row>
     <row r="10">
@@ -642,11 +642,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>395</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -660,16 +660,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>830</v>
       </c>
     </row>
     <row r="12">
@@ -688,11 +688,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>565</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -706,16 +706,16 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>830</v>
+        <v>395</v>
       </c>
     </row>
     <row r="14">
@@ -734,11 +734,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>565</v>
       </c>
     </row>
     <row r="15">
@@ -757,11 +757,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -803,11 +803,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>9150</v>
       </c>
     </row>
     <row r="18">
@@ -826,11 +826,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>3652</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="19">
@@ -867,16 +867,16 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>6352</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -895,11 +895,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>9150</v>
+        <v>3652</v>
       </c>
     </row>
     <row r="22">
@@ -913,16 +913,16 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1037</v>
+        <v>6352</v>
       </c>
     </row>
     <row r="23">
@@ -941,11 +941,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1259</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="24">
@@ -964,11 +964,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25">
@@ -987,11 +987,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26">
@@ -1005,16 +1005,16 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -1028,16 +1028,16 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28">
@@ -1056,11 +1056,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>38</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29">
@@ -1079,11 +1079,11 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -1097,16 +1097,16 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>85</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31">
@@ -1120,16 +1120,16 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>17</v>
+        <v>85</v>
       </c>
     </row>
     <row r="32">
@@ -1148,11 +1148,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33">
@@ -1166,16 +1166,16 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -1189,16 +1189,16 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
     </row>
     <row r="35">
@@ -1217,11 +1217,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>25</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36">
@@ -1281,16 +1281,16 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>223</v>
+        <v>468</v>
       </c>
     </row>
     <row r="39">
@@ -1327,16 +1327,16 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>468</v>
+        <v>223</v>
       </c>
     </row>
     <row r="41">
@@ -1355,11 +1355,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="42">
@@ -1378,11 +1378,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>432</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="43">
@@ -1419,16 +1419,16 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>761</v>
+        <v>432</v>
       </c>
     </row>
     <row r="45">
@@ -1447,11 +1447,11 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>1260</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
@@ -1465,16 +1465,16 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>1092</v>
+        <v>761</v>
       </c>
     </row>
     <row r="47">
@@ -1493,11 +1493,11 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>1335</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="48">
@@ -1516,11 +1516,11 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="49">
@@ -1539,11 +1539,11 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>22</v>
+        <v>39</v>
       </c>
     </row>
     <row r="50">
@@ -1585,11 +1585,11 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -1631,11 +1631,11 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="54">
@@ -1649,16 +1649,16 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>4</v>
+        <v>4428</v>
       </c>
     </row>
     <row r="55">
@@ -1677,11 +1677,11 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>750</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="56">
@@ -1695,16 +1695,16 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>4428</v>
+        <v>629</v>
       </c>
     </row>
     <row r="57">
@@ -1723,11 +1723,11 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>629</v>
+        <v>750</v>
       </c>
     </row>
     <row r="58">
@@ -1746,11 +1746,11 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>1213</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>7</v>
+        <v>109</v>
       </c>
     </row>
     <row r="60">
@@ -1787,16 +1787,16 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>430</v>
+        <v>78</v>
       </c>
     </row>
     <row r="61">
@@ -1810,16 +1810,16 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>109</v>
+        <v>430</v>
       </c>
     </row>
     <row r="62">
@@ -1838,11 +1838,11 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>78</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>119</v>
+        <v>42</v>
       </c>
     </row>
     <row r="65">
@@ -1902,16 +1902,16 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>524</v>
+        <v>41</v>
       </c>
     </row>
     <row r="66">
@@ -1930,11 +1930,11 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>41</v>
+        <v>119</v>
       </c>
     </row>
     <row r="67">
@@ -1948,16 +1948,16 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>42</v>
+        <v>524</v>
       </c>
     </row>
     <row r="68">
@@ -1976,11 +1976,11 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>3</v>
+        <v>2334</v>
       </c>
     </row>
     <row r="69">
@@ -1999,11 +1999,11 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>260</v>
+        <v>1598</v>
       </c>
     </row>
     <row r="70">
@@ -2022,11 +2022,11 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>3507</v>
       </c>
     </row>
     <row r="71">
@@ -2045,11 +2045,11 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>216</v>
+        <v>34063</v>
       </c>
     </row>
     <row r="72">
@@ -2068,11 +2068,11 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>37636</v>
+        <v>886</v>
       </c>
     </row>
     <row r="73">
@@ -2086,16 +2086,16 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>1598</v>
+        <v>37636</v>
       </c>
     </row>
     <row r="74">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>3507</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75">
@@ -2137,11 +2137,11 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>34063</v>
+        <v>260</v>
       </c>
     </row>
     <row r="76">
@@ -2155,16 +2155,16 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>886</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>2334</v>
+        <v>216</v>
       </c>
     </row>
     <row r="78">
@@ -2206,11 +2206,11 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>6</v>
+        <v>162087</v>
       </c>
     </row>
     <row r="79">
@@ -2229,11 +2229,11 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>4338</v>
+        <v>39786</v>
       </c>
     </row>
     <row r="80">
@@ -2247,16 +2247,16 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>22985</v>
+        <v>176905</v>
       </c>
     </row>
     <row r="81">
@@ -2270,16 +2270,16 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>176905</v>
+        <v>15695</v>
       </c>
     </row>
     <row r="82">
@@ -2298,11 +2298,11 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>162087</v>
+        <v>4338</v>
       </c>
     </row>
     <row r="83">
@@ -2321,11 +2321,11 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>39786</v>
+        <v>22985</v>
       </c>
     </row>
     <row r="84">
@@ -2344,11 +2344,11 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>15695</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85">
@@ -2367,11 +2367,11 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>4</v>
+        <v>84</v>
       </c>
     </row>
     <row r="86">
@@ -2390,11 +2390,11 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>159</v>
+        <v>3</v>
       </c>
     </row>
     <row r="87">
@@ -2408,16 +2408,16 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>285</v>
+        <v>7</v>
       </c>
     </row>
     <row r="88">
@@ -2436,11 +2436,11 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>84</v>
+        <v>4</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>3</v>
+        <v>159</v>
       </c>
     </row>
     <row r="90">
@@ -2477,16 +2477,16 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>7</v>
+        <v>285</v>
       </c>
     </row>
     <row r="91">
@@ -2505,11 +2505,11 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>8</v>
+        <v>200</v>
       </c>
     </row>
     <row r="92">
@@ -2528,11 +2528,11 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>55</v>
+        <v>112</v>
       </c>
     </row>
     <row r="93">
@@ -2546,16 +2546,16 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>83</v>
+        <v>55</v>
       </c>
     </row>
     <row r="94">
@@ -2574,11 +2574,11 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>112</v>
+        <v>8</v>
       </c>
     </row>
     <row r="95">
@@ -2592,16 +2592,16 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>200</v>
+        <v>83</v>
       </c>
     </row>
     <row r="96">
@@ -2620,11 +2620,11 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>7</v>
+        <v>516</v>
       </c>
     </row>
     <row r="97">
@@ -2638,16 +2638,16 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
     </row>
     <row r="98">
@@ -2661,16 +2661,16 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>13</v>
+        <v>123</v>
       </c>
     </row>
     <row r="99">
@@ -2689,11 +2689,11 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>516</v>
+        <v>88</v>
       </c>
     </row>
     <row r="100">
@@ -2712,11 +2712,11 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>123</v>
+        <v>7</v>
       </c>
     </row>
     <row r="101">
@@ -2735,11 +2735,11 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>2</v>
+        <v>705</v>
       </c>
     </row>
     <row r="102">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>22</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="103">
@@ -2776,16 +2776,16 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E103" t="n">
-        <v>3052</v>
+        <v>22</v>
       </c>
     </row>
     <row r="104">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>5200</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105">
@@ -2822,16 +2822,16 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>705</v>
+        <v>3052</v>
       </c>
     </row>
     <row r="106">
@@ -2850,11 +2850,11 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="107">
@@ -2868,16 +2868,16 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>87</v>
+        <v>397</v>
       </c>
     </row>
     <row r="108">
@@ -2891,16 +2891,16 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>397</v>
+        <v>81</v>
       </c>
     </row>
     <row r="109">
@@ -2919,11 +2919,11 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="110">
@@ -2942,11 +2942,11 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>6</v>
+        <v>974</v>
       </c>
     </row>
     <row r="111">
@@ -2965,11 +2965,11 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>974</v>
+        <v>4</v>
       </c>
     </row>
     <row r="112">
@@ -2988,11 +2988,11 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>7</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="113">
@@ -3011,11 +3011,11 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>1356</v>
+        <v>817</v>
       </c>
     </row>
     <row r="114">
@@ -3029,16 +3029,16 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>3</v>
+        <v>755</v>
       </c>
     </row>
     <row r="115">
@@ -3052,16 +3052,16 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>755</v>
+        <v>14404</v>
       </c>
     </row>
     <row r="116">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>1014</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="117">
@@ -3103,11 +3103,11 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>817</v>
+        <v>3</v>
       </c>
     </row>
     <row r="118">
@@ -3126,11 +3126,11 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>14404</v>
+        <v>7</v>
       </c>
     </row>
     <row r="119">
@@ -3149,11 +3149,11 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="120">
@@ -3172,11 +3172,11 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>337</v>
+        <v>189</v>
       </c>
     </row>
     <row r="121">
@@ -3190,16 +3190,16 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>135</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="122">
@@ -3213,16 +3213,16 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>1208</v>
+        <v>172</v>
       </c>
     </row>
     <row r="123">
@@ -3241,11 +3241,11 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>3</v>
+        <v>337</v>
       </c>
     </row>
     <row r="124">
@@ -3264,11 +3264,11 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>189</v>
+        <v>135</v>
       </c>
     </row>
     <row r="125">
@@ -3287,11 +3287,11 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>172</v>
+        <v>2</v>
       </c>
     </row>
     <row r="126">
@@ -3310,11 +3310,11 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E126" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E127" t="n">
-        <v>250</v>
+        <v>7</v>
       </c>
     </row>
     <row r="128">
@@ -3379,11 +3379,11 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="130">
@@ -3402,11 +3402,11 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>7</v>
+        <v>250</v>
       </c>
     </row>
     <row r="131">
@@ -3466,16 +3466,16 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E133" t="n">
-        <v>1584</v>
+        <v>701</v>
       </c>
     </row>
     <row r="134">
@@ -3489,16 +3489,16 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>701</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="135">
@@ -3517,11 +3517,11 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E135" t="n">
-        <v>10389</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="136">
@@ -3563,11 +3563,11 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E137" t="n">
-        <v>1332</v>
+        <v>10389</v>
       </c>
     </row>
     <row r="138">
@@ -3581,16 +3581,16 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E138" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="139">
@@ -3604,16 +3604,16 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E139" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="140">
@@ -3701,11 +3701,11 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E143" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
     </row>
     <row r="144">
@@ -3719,16 +3719,16 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="145">
@@ -3747,11 +3747,11 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>13</v>
+        <v>54</v>
       </c>
     </row>
     <row r="146">
@@ -3765,16 +3765,16 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="147">
@@ -3793,11 +3793,11 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148">
@@ -3816,11 +3816,11 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>44</v>
+        <v>4</v>
       </c>
     </row>
     <row r="149">
@@ -3839,11 +3839,11 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="150">
@@ -3862,11 +3862,11 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E150" t="n">
-        <v>4</v>
+        <v>44</v>
       </c>
     </row>
     <row r="151">
@@ -3885,11 +3885,11 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="152">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E152" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="153">
@@ -3931,11 +3931,11 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="154">
@@ -3977,11 +3977,11 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>5</v>
+        <v>85</v>
       </c>
     </row>
     <row r="156">
@@ -4000,11 +4000,11 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E156" t="n">
-        <v>85</v>
+        <v>2</v>
       </c>
     </row>
     <row r="157">
@@ -4023,11 +4023,11 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="158">
@@ -4046,11 +4046,11 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>54</v>
+        <v>10</v>
       </c>
     </row>
     <row r="159">
@@ -4069,11 +4069,11 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E159" t="n">
-        <v>2</v>
+        <v>54</v>
       </c>
     </row>
     <row r="160">
@@ -4092,11 +4092,11 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E160" t="n">
-        <v>687</v>
+        <v>2</v>
       </c>
     </row>
     <row r="161">
@@ -4138,11 +4138,11 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>531</v>
+        <v>58</v>
       </c>
     </row>
     <row r="163">
@@ -4161,11 +4161,11 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>2</v>
+        <v>687</v>
       </c>
     </row>
     <row r="164">
@@ -4184,11 +4184,11 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>58</v>
+        <v>531</v>
       </c>
     </row>
     <row r="165">
@@ -4225,16 +4225,16 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>54</v>
+        <v>13</v>
       </c>
     </row>
     <row r="167">
@@ -4253,11 +4253,11 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E167" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="168">
@@ -4271,16 +4271,16 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>3</v>
+        <v>54</v>
       </c>
     </row>
     <row r="169">
@@ -4299,11 +4299,11 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="170">
@@ -4317,16 +4317,16 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>283</v>
+        <v>2</v>
       </c>
     </row>
     <row r="171">
@@ -4340,16 +4340,16 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E171" t="n">
-        <v>38</v>
+        <v>283</v>
       </c>
     </row>
     <row r="172">
@@ -4368,11 +4368,11 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
     </row>
     <row r="173">
@@ -4391,11 +4391,11 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>2</v>
+        <v>150</v>
       </c>
     </row>
     <row r="174">
@@ -4437,11 +4437,11 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>150</v>
+        <v>58</v>
       </c>
     </row>
     <row r="176">
@@ -4455,16 +4455,16 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E176" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="177">
@@ -4478,16 +4478,16 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E177" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="178">
@@ -4506,11 +4506,11 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
     </row>
     <row r="179">
@@ -4575,11 +4575,11 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>96</v>
+        <v>21</v>
       </c>
     </row>
     <row r="182">
@@ -4621,11 +4621,11 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
     </row>
     <row r="184">
@@ -4662,16 +4662,16 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E185" t="n">
-        <v>387</v>
+        <v>4</v>
       </c>
     </row>
     <row r="186">
@@ -4713,11 +4713,11 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>214</v>
+        <v>206</v>
       </c>
     </row>
     <row r="188">
@@ -4736,11 +4736,11 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>206</v>
+        <v>214</v>
       </c>
     </row>
     <row r="189">
@@ -4754,16 +4754,16 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>4</v>
+        <v>387</v>
       </c>
     </row>
     <row r="190">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
     </row>
     <row r="192">
@@ -4828,11 +4828,11 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>48</v>
+        <v>120</v>
       </c>
     </row>
     <row r="193">
@@ -4851,11 +4851,11 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
     </row>
     <row r="194">
@@ -4874,11 +4874,11 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="195">
@@ -4892,12 +4892,12 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E195" t="n">
@@ -4920,11 +4920,11 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="197">
@@ -4943,11 +4943,11 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="198">
@@ -4961,12 +4961,12 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -4989,11 +4989,11 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="200">
@@ -5012,11 +5012,11 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>101</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E202" t="n">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E203" t="n">
@@ -5122,16 +5122,16 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="206">
@@ -5150,11 +5150,11 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207">
@@ -5168,16 +5168,16 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="208">
@@ -5196,11 +5196,11 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="209">
@@ -5237,16 +5237,16 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>147</v>
+        <v>104</v>
       </c>
     </row>
     <row r="211">
@@ -5265,11 +5265,11 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>104</v>
+        <v>44</v>
       </c>
     </row>
     <row r="212">
@@ -5288,11 +5288,11 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
     </row>
     <row r="213">
@@ -5311,11 +5311,11 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>23</v>
+        <v>68</v>
       </c>
     </row>
     <row r="214">
@@ -5352,16 +5352,16 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E215" t="n">
-        <v>68</v>
+        <v>147</v>
       </c>
     </row>
     <row r="216">
@@ -5375,16 +5375,16 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E216" t="n">
-        <v>63</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217">
@@ -5403,11 +5403,11 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E217" t="n">
-        <v>21</v>
+        <v>43</v>
       </c>
     </row>
     <row r="218">
@@ -5444,16 +5444,16 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E219" t="n">
-        <v>3</v>
+        <v>63</v>
       </c>
     </row>
     <row r="220">
@@ -5472,11 +5472,11 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E220" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="221">
@@ -5495,11 +5495,11 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E221" t="n">
-        <v>43</v>
+        <v>3</v>
       </c>
     </row>
     <row r="222">
@@ -5518,11 +5518,11 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E222" t="n">
-        <v>25</v>
+        <v>83</v>
       </c>
     </row>
     <row r="223">
@@ -5541,11 +5541,11 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E223" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="224">
@@ -5564,11 +5564,11 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E224" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="225">
@@ -5587,11 +5587,11 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E225" t="n">
-        <v>83</v>
+        <v>25</v>
       </c>
     </row>
     <row r="226">
@@ -5909,11 +5909,11 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>165</v>
+        <v>250</v>
       </c>
     </row>
     <row r="240">
@@ -5932,11 +5932,11 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E240" t="n">
-        <v>250</v>
+        <v>165</v>
       </c>
     </row>
     <row r="241">
@@ -5955,11 +5955,11 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E241" t="n">
-        <v>199</v>
+        <v>1</v>
       </c>
     </row>
     <row r="242">
@@ -5978,11 +5978,11 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E242" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="243">
@@ -6001,11 +6001,11 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E243" t="n">
-        <v>20</v>
+        <v>199</v>
       </c>
     </row>
     <row r="244">
@@ -6019,16 +6019,16 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>1482</v>
+        <v>3963</v>
       </c>
     </row>
     <row r="245">
@@ -6047,11 +6047,11 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>944</v>
+        <v>3879</v>
       </c>
     </row>
     <row r="246">
@@ -6065,16 +6065,16 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E246" t="n">
-        <v>3963</v>
+        <v>944</v>
       </c>
     </row>
     <row r="247">
@@ -6093,11 +6093,11 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E247" t="n">
-        <v>2</v>
+        <v>4103</v>
       </c>
     </row>
     <row r="248">
@@ -6116,11 +6116,11 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E248" t="n">
-        <v>3879</v>
+        <v>2</v>
       </c>
     </row>
     <row r="249">
@@ -6162,11 +6162,11 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>4103</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="251">
@@ -6180,16 +6180,16 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="252">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="253">
@@ -6249,16 +6249,16 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="255">
@@ -6277,11 +6277,11 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>477</v>
+        <v>283</v>
       </c>
     </row>
     <row r="256">
@@ -6300,11 +6300,11 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>29</v>
+        <v>477</v>
       </c>
     </row>
     <row r="257">
@@ -6323,11 +6323,11 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>283</v>
+        <v>547</v>
       </c>
     </row>
     <row r="258">
@@ -6369,11 +6369,11 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>547</v>
+        <v>29</v>
       </c>
     </row>
     <row r="260">
@@ -6410,16 +6410,16 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>1072</v>
+        <v>423</v>
       </c>
     </row>
     <row r="262">
@@ -6433,16 +6433,16 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E262" t="n">
-        <v>423</v>
+        <v>854</v>
       </c>
     </row>
     <row r="263">
@@ -6484,11 +6484,11 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>854</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="265">
@@ -6553,11 +6553,11 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>93</v>
+        <v>468</v>
       </c>
     </row>
     <row r="268">
@@ -6576,11 +6576,11 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>468</v>
+        <v>93</v>
       </c>
     </row>
     <row r="269">
@@ -6599,11 +6599,11 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>434</v>
+        <v>343</v>
       </c>
     </row>
     <row r="270">
@@ -6622,11 +6622,11 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>256</v>
+        <v>434</v>
       </c>
     </row>
     <row r="271">
@@ -6663,16 +6663,16 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>202</v>
+        <v>256</v>
       </c>
     </row>
     <row r="273">
@@ -6686,16 +6686,16 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>343</v>
+        <v>202</v>
       </c>
     </row>
     <row r="274">
@@ -6709,16 +6709,16 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>4</v>
+        <v>149</v>
       </c>
     </row>
     <row r="275">
@@ -6732,16 +6732,16 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>149</v>
+        <v>115</v>
       </c>
     </row>
     <row r="276">
@@ -6760,11 +6760,11 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
     </row>
     <row r="277">
@@ -6783,11 +6783,11 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>115</v>
+        <v>4</v>
       </c>
     </row>
     <row r="278">
@@ -6806,11 +6806,11 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
     </row>
     <row r="279">
@@ -6824,16 +6824,16 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>60</v>
+        <v>317</v>
       </c>
     </row>
     <row r="280">
@@ -6852,11 +6852,11 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>25</v>
+        <v>143</v>
       </c>
     </row>
     <row r="281">
@@ -6875,11 +6875,11 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>143</v>
+        <v>25</v>
       </c>
     </row>
     <row r="282">
@@ -6898,11 +6898,11 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>7</v>
+        <v>60</v>
       </c>
     </row>
     <row r="283">
@@ -6921,11 +6921,11 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>1674</v>
+        <v>7</v>
       </c>
     </row>
     <row r="284">
@@ -6939,16 +6939,16 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>317</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="285">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E285" t="n">
@@ -7013,11 +7013,11 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="288">
@@ -7036,11 +7036,11 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="289">
@@ -7054,16 +7054,16 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>858</v>
+        <v>538</v>
       </c>
     </row>
     <row r="290">
@@ -7082,11 +7082,11 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>4</v>
+        <v>858</v>
       </c>
     </row>
     <row r="291">
@@ -7105,11 +7105,11 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>16</v>
+        <v>38</v>
       </c>
     </row>
     <row r="292">
@@ -7128,11 +7128,11 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>38</v>
+        <v>297</v>
       </c>
     </row>
     <row r="293">
@@ -7146,16 +7146,16 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>538</v>
+        <v>4</v>
       </c>
     </row>
     <row r="294">
@@ -7174,11 +7174,11 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>297</v>
+        <v>16</v>
       </c>
     </row>
     <row r="295">
@@ -7220,11 +7220,11 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>87</v>
+        <v>15</v>
       </c>
     </row>
     <row r="297">
@@ -7266,11 +7266,11 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>15</v>
+        <v>87</v>
       </c>
     </row>
     <row r="299">
@@ -7289,11 +7289,11 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
     </row>
     <row r="300">
@@ -7312,11 +7312,11 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="301">
@@ -7335,11 +7335,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
     </row>
     <row r="302">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="303">
@@ -7381,11 +7381,11 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>48</v>
+        <v>66</v>
       </c>
     </row>
     <row r="304">
@@ -7404,11 +7404,11 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
     </row>
     <row r="305">
@@ -7427,11 +7427,11 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>66</v>
+        <v>3</v>
       </c>
     </row>
     <row r="306">

</xml_diff>

<commit_message>
atualizacao volumes para LOA 2024
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -458,11 +458,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>500</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -481,11 +481,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>34</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
@@ -504,11 +504,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>78</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -550,11 +550,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>2733</v>
       </c>
     </row>
     <row r="7">
@@ -573,11 +573,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>73</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -596,11 +596,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>14</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9">
@@ -619,11 +619,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2733</v>
+        <v>500</v>
       </c>
     </row>
     <row r="10">
@@ -642,11 +642,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>395</v>
       </c>
     </row>
     <row r="11">
@@ -660,16 +660,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>830</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -688,11 +688,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>14</v>
+        <v>565</v>
       </c>
     </row>
     <row r="13">
@@ -706,16 +706,16 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>395</v>
+        <v>830</v>
       </c>
     </row>
     <row r="14">
@@ -734,11 +734,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>565</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -757,11 +757,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
@@ -803,11 +803,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>9150</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
@@ -826,11 +826,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1259</v>
+        <v>3652</v>
       </c>
     </row>
     <row r="19">
@@ -867,16 +867,16 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>6352</v>
       </c>
     </row>
     <row r="21">
@@ -895,11 +895,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>3652</v>
+        <v>9150</v>
       </c>
     </row>
     <row r="22">
@@ -913,16 +913,16 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>6352</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="23">
@@ -941,11 +941,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1037</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="24">
@@ -964,11 +964,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -987,11 +987,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>38</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26">
@@ -1005,16 +1005,16 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27">
@@ -1028,16 +1028,16 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -1056,11 +1056,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29">
@@ -1079,11 +1079,11 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30">
@@ -1097,16 +1097,16 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>17</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31">
@@ -1120,16 +1120,16 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>85</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32">
@@ -1148,11 +1148,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -1166,16 +1166,16 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
     </row>
     <row r="34">
@@ -1189,16 +1189,16 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35">
@@ -1217,11 +1217,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>64</v>
+        <v>25</v>
       </c>
     </row>
     <row r="36">
@@ -1281,16 +1281,16 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>468</v>
+        <v>223</v>
       </c>
     </row>
     <row r="39">
@@ -1327,16 +1327,16 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>223</v>
+        <v>468</v>
       </c>
     </row>
     <row r="41">
@@ -1355,11 +1355,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1260</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
@@ -1378,11 +1378,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1335</v>
+        <v>432</v>
       </c>
     </row>
     <row r="43">
@@ -1419,16 +1419,16 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>432</v>
+        <v>761</v>
       </c>
     </row>
     <row r="45">
@@ -1447,11 +1447,11 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>6</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="46">
@@ -1465,16 +1465,16 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>761</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="47">
@@ -1493,11 +1493,11 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>1092</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="48">
@@ -1516,11 +1516,11 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -1539,11 +1539,11 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>39</v>
+        <v>22</v>
       </c>
     </row>
     <row r="50">
@@ -1585,11 +1585,11 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="52">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
     </row>
     <row r="53">
@@ -1631,11 +1631,11 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="54">
@@ -1649,16 +1649,16 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>4428</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55">
@@ -1677,11 +1677,11 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>1213</v>
+        <v>750</v>
       </c>
     </row>
     <row r="56">
@@ -1695,16 +1695,16 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>629</v>
+        <v>4428</v>
       </c>
     </row>
     <row r="57">
@@ -1723,11 +1723,11 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>750</v>
+        <v>629</v>
       </c>
     </row>
     <row r="58">
@@ -1746,11 +1746,11 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>4</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="59">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>109</v>
+        <v>7</v>
       </c>
     </row>
     <row r="60">
@@ -1787,16 +1787,16 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>78</v>
+        <v>430</v>
       </c>
     </row>
     <row r="61">
@@ -1810,16 +1810,16 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>430</v>
+        <v>109</v>
       </c>
     </row>
     <row r="62">
@@ -1838,11 +1838,11 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>7</v>
+        <v>78</v>
       </c>
     </row>
     <row r="63">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>42</v>
+        <v>119</v>
       </c>
     </row>
     <row r="65">
@@ -1902,16 +1902,16 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>41</v>
+        <v>524</v>
       </c>
     </row>
     <row r="66">
@@ -1930,11 +1930,11 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>119</v>
+        <v>41</v>
       </c>
     </row>
     <row r="67">
@@ -1948,16 +1948,16 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>524</v>
+        <v>42</v>
       </c>
     </row>
     <row r="68">
@@ -1976,11 +1976,11 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>2334</v>
+        <v>3</v>
       </c>
     </row>
     <row r="69">
@@ -1999,11 +1999,11 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>1598</v>
+        <v>260</v>
       </c>
     </row>
     <row r="70">
@@ -2022,11 +2022,11 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>3507</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71">
@@ -2045,11 +2045,11 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>34063</v>
+        <v>216</v>
       </c>
     </row>
     <row r="72">
@@ -2068,11 +2068,11 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>886</v>
+        <v>37636</v>
       </c>
     </row>
     <row r="73">
@@ -2086,16 +2086,16 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>37636</v>
+        <v>1598</v>
       </c>
     </row>
     <row r="74">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>3</v>
+        <v>3507</v>
       </c>
     </row>
     <row r="75">
@@ -2137,11 +2137,11 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>260</v>
+        <v>34063</v>
       </c>
     </row>
     <row r="76">
@@ -2155,16 +2155,16 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>2</v>
+        <v>886</v>
       </c>
     </row>
     <row r="77">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>216</v>
+        <v>2334</v>
       </c>
     </row>
     <row r="78">
@@ -2206,11 +2206,11 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>162087</v>
+        <v>6</v>
       </c>
     </row>
     <row r="79">
@@ -2229,11 +2229,11 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>39786</v>
+        <v>4338</v>
       </c>
     </row>
     <row r="80">
@@ -2247,16 +2247,16 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>176905</v>
+        <v>22985</v>
       </c>
     </row>
     <row r="81">
@@ -2270,16 +2270,16 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>15695</v>
+        <v>176905</v>
       </c>
     </row>
     <row r="82">
@@ -2298,11 +2298,11 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>4338</v>
+        <v>162087</v>
       </c>
     </row>
     <row r="83">
@@ -2321,11 +2321,11 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>22985</v>
+        <v>39786</v>
       </c>
     </row>
     <row r="84">
@@ -2344,11 +2344,11 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>6</v>
+        <v>15695</v>
       </c>
     </row>
     <row r="85">
@@ -2367,11 +2367,11 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>84</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86">
@@ -2390,11 +2390,11 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>3</v>
+        <v>159</v>
       </c>
     </row>
     <row r="87">
@@ -2408,16 +2408,16 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>7</v>
+        <v>285</v>
       </c>
     </row>
     <row r="88">
@@ -2436,11 +2436,11 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>4</v>
+        <v>84</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>159</v>
+        <v>3</v>
       </c>
     </row>
     <row r="90">
@@ -2477,16 +2477,16 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>285</v>
+        <v>7</v>
       </c>
     </row>
     <row r="91">
@@ -2505,11 +2505,11 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>200</v>
+        <v>8</v>
       </c>
     </row>
     <row r="92">
@@ -2528,11 +2528,11 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>112</v>
+        <v>55</v>
       </c>
     </row>
     <row r="93">
@@ -2551,11 +2551,11 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>55</v>
+        <v>200</v>
       </c>
     </row>
     <row r="94">
@@ -2574,11 +2574,11 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>8</v>
+        <v>112</v>
       </c>
     </row>
     <row r="95">
@@ -2620,11 +2620,11 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>516</v>
+        <v>123</v>
       </c>
     </row>
     <row r="97">
@@ -2666,11 +2666,11 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>123</v>
+        <v>7</v>
       </c>
     </row>
     <row r="99">
@@ -2689,11 +2689,11 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>88</v>
+        <v>516</v>
       </c>
     </row>
     <row r="100">
@@ -2712,11 +2712,11 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>7</v>
+        <v>88</v>
       </c>
     </row>
     <row r="101">
@@ -2730,16 +2730,16 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>705</v>
+        <v>3052</v>
       </c>
     </row>
     <row r="102">
@@ -2781,11 +2781,11 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E103" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="105">
@@ -2822,16 +2822,16 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>3052</v>
+        <v>705</v>
       </c>
     </row>
     <row r="106">
@@ -2850,11 +2850,11 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="107">
@@ -2868,16 +2868,16 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>397</v>
+        <v>81</v>
       </c>
     </row>
     <row r="108">
@@ -2891,16 +2891,16 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>81</v>
+        <v>397</v>
       </c>
     </row>
     <row r="109">
@@ -2919,11 +2919,11 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>87</v>
+        <v>6</v>
       </c>
     </row>
     <row r="110">
@@ -2965,11 +2965,11 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>4</v>
+        <v>87</v>
       </c>
     </row>
     <row r="112">
@@ -2988,11 +2988,11 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>1014</v>
+        <v>7</v>
       </c>
     </row>
     <row r="113">
@@ -3011,11 +3011,11 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>817</v>
+        <v>14404</v>
       </c>
     </row>
     <row r="114">
@@ -3029,16 +3029,16 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>755</v>
+        <v>817</v>
       </c>
     </row>
     <row r="115">
@@ -3057,11 +3057,11 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>14404</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="116">
@@ -3075,16 +3075,16 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>1356</v>
+        <v>755</v>
       </c>
     </row>
     <row r="117">
@@ -3103,11 +3103,11 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>3</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="118">
@@ -3126,11 +3126,11 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="119">
@@ -3149,11 +3149,11 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>3</v>
+        <v>135</v>
       </c>
     </row>
     <row r="120">
@@ -3167,16 +3167,16 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>189</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="121">
@@ -3190,16 +3190,16 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>1208</v>
+        <v>337</v>
       </c>
     </row>
     <row r="122">
@@ -3241,11 +3241,11 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>337</v>
+        <v>2</v>
       </c>
     </row>
     <row r="124">
@@ -3264,11 +3264,11 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>135</v>
+        <v>189</v>
       </c>
     </row>
     <row r="125">
@@ -3287,11 +3287,11 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="126">
@@ -3310,11 +3310,11 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E126" t="n">
-        <v>30</v>
+        <v>250</v>
       </c>
     </row>
     <row r="127">
@@ -3351,16 +3351,16 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E128" t="n">
-        <v>52</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="129">
@@ -3402,11 +3402,11 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>250</v>
+        <v>30</v>
       </c>
     </row>
     <row r="131">
@@ -3420,16 +3420,16 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E131" t="n">
-        <v>1117</v>
+        <v>52</v>
       </c>
     </row>
     <row r="132">
@@ -3448,11 +3448,11 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E132" t="n">
-        <v>726</v>
+        <v>701</v>
       </c>
     </row>
     <row r="133">
@@ -3466,16 +3466,16 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E133" t="n">
-        <v>701</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="134">
@@ -3489,16 +3489,16 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>1584</v>
+        <v>726</v>
       </c>
     </row>
     <row r="135">
@@ -3517,11 +3517,11 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E135" t="n">
-        <v>1332</v>
+        <v>10389</v>
       </c>
     </row>
     <row r="136">
@@ -3535,16 +3535,16 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E136" t="n">
-        <v>7508</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="137">
@@ -3558,16 +3558,16 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E137" t="n">
-        <v>10389</v>
+        <v>7508</v>
       </c>
     </row>
     <row r="138">
@@ -3586,11 +3586,11 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E138" t="n">
-        <v>21</v>
+        <v>140</v>
       </c>
     </row>
     <row r="139">
@@ -3604,16 +3604,16 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E139" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="140">
@@ -3632,11 +3632,11 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E140" t="n">
-        <v>140</v>
+        <v>21</v>
       </c>
     </row>
     <row r="141">
@@ -3673,16 +3673,16 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E142" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="143">
@@ -3719,16 +3719,16 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>11</v>
+        <v>54</v>
       </c>
     </row>
     <row r="145">
@@ -3747,11 +3747,11 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>54</v>
+        <v>13</v>
       </c>
     </row>
     <row r="146">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147">
@@ -3788,16 +3788,16 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="148">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E148" t="n">
@@ -3839,11 +3839,11 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="150">
@@ -3862,11 +3862,11 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E150" t="n">
-        <v>44</v>
+        <v>3</v>
       </c>
     </row>
     <row r="151">
@@ -3885,11 +3885,11 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="152">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E152" t="n">
-        <v>2</v>
+        <v>44</v>
       </c>
     </row>
     <row r="153">
@@ -3931,11 +3931,11 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="154">
@@ -3954,11 +3954,11 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>2</v>
+        <v>85</v>
       </c>
     </row>
     <row r="155">
@@ -3977,11 +3977,11 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>85</v>
+        <v>5</v>
       </c>
     </row>
     <row r="156">
@@ -4000,7 +4000,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -4023,11 +4023,11 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="158">
@@ -4046,11 +4046,11 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>10</v>
+        <v>54</v>
       </c>
     </row>
     <row r="159">
@@ -4069,11 +4069,11 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E159" t="n">
-        <v>54</v>
+        <v>2</v>
       </c>
     </row>
     <row r="160">
@@ -4087,16 +4087,16 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E160" t="n">
-        <v>2</v>
+        <v>3362</v>
       </c>
     </row>
     <row r="161">
@@ -4115,11 +4115,11 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E161" t="n">
-        <v>964</v>
+        <v>531</v>
       </c>
     </row>
     <row r="162">
@@ -4161,11 +4161,11 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>687</v>
+        <v>964</v>
       </c>
     </row>
     <row r="164">
@@ -4184,11 +4184,11 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>531</v>
+        <v>2</v>
       </c>
     </row>
     <row r="165">
@@ -4202,16 +4202,16 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>3362</v>
+        <v>687</v>
       </c>
     </row>
     <row r="166">
@@ -4253,11 +4253,11 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E167" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="168">
@@ -4271,16 +4271,16 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>54</v>
+        <v>3</v>
       </c>
     </row>
     <row r="169">
@@ -4294,16 +4294,16 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>4</v>
+        <v>54</v>
       </c>
     </row>
     <row r="170">
@@ -4317,16 +4317,16 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>2</v>
+        <v>283</v>
       </c>
     </row>
     <row r="171">
@@ -4340,16 +4340,16 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E171" t="n">
-        <v>283</v>
+        <v>38</v>
       </c>
     </row>
     <row r="172">
@@ -4368,11 +4368,11 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>38</v>
+        <v>58</v>
       </c>
     </row>
     <row r="173">
@@ -4391,11 +4391,11 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>150</v>
+        <v>2</v>
       </c>
     </row>
     <row r="174">
@@ -4437,11 +4437,11 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>58</v>
+        <v>150</v>
       </c>
     </row>
     <row r="176">
@@ -4455,16 +4455,16 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E176" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="177">
@@ -4478,16 +4478,16 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E177" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="178">
@@ -4506,11 +4506,11 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="179">
@@ -4575,11 +4575,11 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
     </row>
     <row r="182">
@@ -4621,11 +4621,11 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>96</v>
+        <v>21</v>
       </c>
     </row>
     <row r="184">
@@ -4662,16 +4662,16 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E185" t="n">
-        <v>4</v>
+        <v>387</v>
       </c>
     </row>
     <row r="186">
@@ -4713,11 +4713,11 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>206</v>
+        <v>214</v>
       </c>
     </row>
     <row r="188">
@@ -4736,11 +4736,11 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>214</v>
+        <v>206</v>
       </c>
     </row>
     <row r="189">
@@ -4754,16 +4754,16 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>387</v>
+        <v>4</v>
       </c>
     </row>
     <row r="190">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>4</v>
+        <v>38</v>
       </c>
     </row>
     <row r="192">
@@ -4828,11 +4828,11 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>120</v>
+        <v>48</v>
       </c>
     </row>
     <row r="193">
@@ -4851,11 +4851,11 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
     </row>
     <row r="194">
@@ -4874,11 +4874,11 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="195">
@@ -4892,12 +4892,12 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E195" t="n">
@@ -4920,11 +4920,11 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="197">
@@ -4943,11 +4943,11 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="198">
@@ -4961,12 +4961,12 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -4989,11 +4989,11 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="200">
@@ -5012,11 +5012,11 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>1</v>
+        <v>101</v>
       </c>
     </row>
     <row r="201">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E202" t="n">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E203" t="n">
@@ -5122,16 +5122,16 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="206">
@@ -5150,11 +5150,11 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="207">
@@ -5168,16 +5168,16 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
     </row>
     <row r="208">
@@ -5196,11 +5196,11 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="209">
@@ -5237,16 +5237,16 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>104</v>
+        <v>147</v>
       </c>
     </row>
     <row r="211">
@@ -5265,11 +5265,11 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>44</v>
+        <v>104</v>
       </c>
     </row>
     <row r="212">
@@ -5288,11 +5288,11 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>23</v>
+        <v>44</v>
       </c>
     </row>
     <row r="213">
@@ -5311,11 +5311,11 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>68</v>
+        <v>23</v>
       </c>
     </row>
     <row r="214">
@@ -5352,16 +5352,16 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E215" t="n">
-        <v>147</v>
+        <v>68</v>
       </c>
     </row>
     <row r="216">
@@ -5375,16 +5375,16 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E216" t="n">
-        <v>1</v>
+        <v>63</v>
       </c>
     </row>
     <row r="217">
@@ -5403,11 +5403,11 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E217" t="n">
-        <v>43</v>
+        <v>21</v>
       </c>
     </row>
     <row r="218">
@@ -5444,16 +5444,16 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E219" t="n">
-        <v>63</v>
+        <v>3</v>
       </c>
     </row>
     <row r="220">
@@ -5472,11 +5472,11 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E220" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="221">
@@ -5495,11 +5495,11 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E221" t="n">
-        <v>3</v>
+        <v>43</v>
       </c>
     </row>
     <row r="222">
@@ -5518,11 +5518,11 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E222" t="n">
-        <v>83</v>
+        <v>25</v>
       </c>
     </row>
     <row r="223">
@@ -5541,11 +5541,11 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E223" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="224">
@@ -5564,11 +5564,11 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E224" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="225">
@@ -5587,11 +5587,11 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E225" t="n">
-        <v>25</v>
+        <v>83</v>
       </c>
     </row>
     <row r="226">
@@ -5932,11 +5932,11 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E240" t="n">
-        <v>165</v>
+        <v>199</v>
       </c>
     </row>
     <row r="241">
@@ -6001,11 +6001,11 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E243" t="n">
-        <v>199</v>
+        <v>165</v>
       </c>
     </row>
     <row r="244">
@@ -6019,16 +6019,16 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>3963</v>
+        <v>587</v>
       </c>
     </row>
     <row r="245">
@@ -6047,11 +6047,11 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>3879</v>
+        <v>944</v>
       </c>
     </row>
     <row r="246">
@@ -6070,11 +6070,11 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E246" t="n">
-        <v>944</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="247">
@@ -6093,11 +6093,11 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E247" t="n">
-        <v>4103</v>
+        <v>3879</v>
       </c>
     </row>
     <row r="248">
@@ -6134,16 +6134,16 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E249" t="n">
-        <v>587</v>
+        <v>3963</v>
       </c>
     </row>
     <row r="250">
@@ -6162,11 +6162,11 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>1482</v>
+        <v>4103</v>
       </c>
     </row>
     <row r="251">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="253">
@@ -6231,11 +6231,11 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E253" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="254">
@@ -6254,11 +6254,11 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="255">
@@ -6295,16 +6295,16 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>477</v>
+        <v>5893</v>
       </c>
     </row>
     <row r="257">
@@ -6346,11 +6346,11 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E258" t="n">
-        <v>12</v>
+        <v>29</v>
       </c>
     </row>
     <row r="259">
@@ -6369,11 +6369,11 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>29</v>
+        <v>12</v>
       </c>
     </row>
     <row r="260">
@@ -6387,16 +6387,16 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>5893</v>
+        <v>477</v>
       </c>
     </row>
     <row r="261">
@@ -6410,16 +6410,16 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>423</v>
+        <v>106</v>
       </c>
     </row>
     <row r="262">
@@ -6438,11 +6438,11 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E262" t="n">
-        <v>854</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="263">
@@ -6461,11 +6461,11 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E263" t="n">
-        <v>106</v>
+        <v>277</v>
       </c>
     </row>
     <row r="264">
@@ -6484,11 +6484,11 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>1072</v>
+        <v>2</v>
       </c>
     </row>
     <row r="265">
@@ -6507,11 +6507,11 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E265" t="n">
-        <v>2</v>
+        <v>854</v>
       </c>
     </row>
     <row r="266">
@@ -6525,16 +6525,16 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>277</v>
+        <v>423</v>
       </c>
     </row>
     <row r="267">
@@ -6599,11 +6599,11 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>343</v>
+        <v>434</v>
       </c>
     </row>
     <row r="270">
@@ -6622,11 +6622,11 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>434</v>
+        <v>256</v>
       </c>
     </row>
     <row r="271">
@@ -6663,16 +6663,16 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>256</v>
+        <v>202</v>
       </c>
     </row>
     <row r="273">
@@ -6686,16 +6686,16 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>202</v>
+        <v>343</v>
       </c>
     </row>
     <row r="274">
@@ -6709,16 +6709,16 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>149</v>
+        <v>18</v>
       </c>
     </row>
     <row r="275">
@@ -6737,11 +6737,11 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>115</v>
+        <v>4</v>
       </c>
     </row>
     <row r="276">
@@ -6760,11 +6760,11 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>4</v>
+        <v>115</v>
       </c>
     </row>
     <row r="277">
@@ -6778,16 +6778,16 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>4</v>
+        <v>149</v>
       </c>
     </row>
     <row r="278">
@@ -6806,11 +6806,11 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
     </row>
     <row r="279">
@@ -6824,16 +6824,16 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>317</v>
+        <v>143</v>
       </c>
     </row>
     <row r="280">
@@ -6852,11 +6852,11 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>143</v>
+        <v>60</v>
       </c>
     </row>
     <row r="281">
@@ -6875,11 +6875,11 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="282">
@@ -6898,11 +6898,11 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
     </row>
     <row r="283">
@@ -6916,16 +6916,16 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>7</v>
+        <v>317</v>
       </c>
     </row>
     <row r="284">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E285" t="n">
@@ -6990,11 +6990,11 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="287">
@@ -7013,7 +7013,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E287" t="n">
@@ -7036,11 +7036,11 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="289">
@@ -7054,16 +7054,16 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>538</v>
+        <v>4</v>
       </c>
     </row>
     <row r="290">
@@ -7105,11 +7105,11 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>38</v>
+        <v>297</v>
       </c>
     </row>
     <row r="292">
@@ -7128,11 +7128,11 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>297</v>
+        <v>38</v>
       </c>
     </row>
     <row r="293">
@@ -7146,16 +7146,16 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>4</v>
+        <v>538</v>
       </c>
     </row>
     <row r="294">
@@ -7192,16 +7192,16 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
     </row>
     <row r="296">
@@ -7220,11 +7220,11 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="297">
@@ -7243,11 +7243,11 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>9</v>
+        <v>87</v>
       </c>
     </row>
     <row r="298">
@@ -7261,16 +7261,16 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>87</v>
+        <v>33</v>
       </c>
     </row>
     <row r="299">
@@ -7289,11 +7289,11 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="300">
@@ -7312,11 +7312,11 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="301">
@@ -7335,11 +7335,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="302">
@@ -7381,11 +7381,11 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>66</v>
+        <v>3</v>
       </c>
     </row>
     <row r="304">
@@ -7404,11 +7404,11 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>48</v>
+        <v>66</v>
       </c>
     </row>
     <row r="305">
@@ -7427,11 +7427,11 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
     </row>
     <row r="306">
@@ -7657,11 +7657,11 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E315" t="n">
-        <v>188</v>
+        <v>318</v>
       </c>
     </row>
     <row r="316">
@@ -7680,11 +7680,11 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E316" t="n">
-        <v>318</v>
+        <v>188</v>
       </c>
     </row>
     <row r="317">
@@ -7726,11 +7726,11 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E318" t="n">
-        <v>7</v>
+        <v>43</v>
       </c>
     </row>
     <row r="319">
@@ -7749,11 +7749,11 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E319" t="n">
-        <v>47</v>
+        <v>12</v>
       </c>
     </row>
     <row r="320">
@@ -7772,11 +7772,11 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E320" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="321">
@@ -7795,11 +7795,11 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E321" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="322">

</xml_diff>

<commit_message>
chore(bancos): atualiza bancos ploa 2025
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -3908,11 +3908,11 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E152" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
     </row>
     <row r="153">
@@ -3931,11 +3931,11 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
     </row>
     <row r="154">
@@ -3977,11 +3977,11 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>88</v>
+        <v>2</v>
       </c>
     </row>
     <row r="156">
@@ -4000,11 +4000,11 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E156" t="n">
-        <v>2</v>
+        <v>88</v>
       </c>
     </row>
     <row r="157">
@@ -4023,11 +4023,11 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>61</v>
+        <v>9</v>
       </c>
     </row>
     <row r="158">
@@ -4069,11 +4069,11 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E159" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="160">
@@ -4092,11 +4092,11 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E160" t="n">
-        <v>3</v>
+        <v>61</v>
       </c>
     </row>
     <row r="161">
@@ -4115,11 +4115,11 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E161" t="n">
-        <v>528</v>
+        <v>917</v>
       </c>
     </row>
     <row r="162">
@@ -4138,11 +4138,11 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>917</v>
+        <v>75</v>
       </c>
     </row>
     <row r="163">
@@ -4161,11 +4161,11 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>75</v>
+        <v>907</v>
       </c>
     </row>
     <row r="164">
@@ -4184,11 +4184,11 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>907</v>
+        <v>528</v>
       </c>
     </row>
     <row r="165">
@@ -4202,16 +4202,16 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>2</v>
+        <v>3286</v>
       </c>
     </row>
     <row r="166">
@@ -4225,16 +4225,16 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>3286</v>
+        <v>2</v>
       </c>
     </row>
     <row r="167">
@@ -4248,16 +4248,16 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E167" t="n">
-        <v>3</v>
+        <v>54</v>
       </c>
     </row>
     <row r="168">
@@ -4317,16 +4317,16 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>54</v>
+        <v>3</v>
       </c>
     </row>
     <row r="171">
@@ -4506,11 +4506,11 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
     </row>
     <row r="179">
@@ -4529,11 +4529,11 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E179" t="n">
-        <v>3</v>
+        <v>58</v>
       </c>
     </row>
     <row r="180">
@@ -4575,11 +4575,11 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>58</v>
+        <v>24</v>
       </c>
     </row>
     <row r="182">
@@ -4593,16 +4593,16 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>94</v>
+        <v>281</v>
       </c>
     </row>
     <row r="183">
@@ -4621,11 +4621,11 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>77</v>
+        <v>53</v>
       </c>
     </row>
     <row r="184">
@@ -4639,16 +4639,16 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E184" t="n">
-        <v>281</v>
+        <v>94</v>
       </c>
     </row>
     <row r="185">
@@ -4690,11 +4690,11 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E186" t="n">
-        <v>53</v>
+        <v>77</v>
       </c>
     </row>
     <row r="187">
@@ -4713,11 +4713,11 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>266</v>
+        <v>262</v>
       </c>
     </row>
     <row r="188">
@@ -4736,11 +4736,11 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>1</v>
+        <v>266</v>
       </c>
     </row>
     <row r="189">
@@ -4759,11 +4759,11 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>262</v>
+        <v>1</v>
       </c>
     </row>
     <row r="190">
@@ -4874,11 +4874,11 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="195">
@@ -4897,11 +4897,11 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E195" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="196">
@@ -4938,16 +4938,16 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>24</v>
+        <v>50</v>
       </c>
     </row>
     <row r="198">
@@ -4966,11 +4966,11 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E198" t="n">
-        <v>284</v>
+        <v>1</v>
       </c>
     </row>
     <row r="199">
@@ -4984,16 +4984,16 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="200">
@@ -5012,11 +5012,11 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>1</v>
+        <v>284</v>
       </c>
     </row>
     <row r="201">
@@ -5035,11 +5035,11 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E201" t="n">
-        <v>49</v>
+        <v>23</v>
       </c>
     </row>
     <row r="202">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E202" t="n">
-        <v>23</v>
+        <v>213</v>
       </c>
     </row>
     <row r="203">
@@ -5081,11 +5081,11 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E203" t="n">
-        <v>213</v>
+        <v>24</v>
       </c>
     </row>
     <row r="204">
@@ -5099,16 +5099,16 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E204" t="n">
-        <v>2</v>
+        <v>81</v>
       </c>
     </row>
     <row r="205">
@@ -5145,16 +5145,16 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>81</v>
+        <v>42</v>
       </c>
     </row>
     <row r="207">
@@ -5173,11 +5173,11 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208">
@@ -5214,16 +5214,16 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E209" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="210">
@@ -5242,11 +5242,11 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
     </row>
     <row r="211">
@@ -5265,11 +5265,11 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="212">
@@ -5283,16 +5283,16 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="213">
@@ -5311,11 +5311,11 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
     </row>
     <row r="214">
@@ -5329,16 +5329,16 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E214" t="n">
-        <v>102</v>
+        <v>135</v>
       </c>
     </row>
     <row r="215">
@@ -5357,11 +5357,11 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E215" t="n">
-        <v>48</v>
+        <v>102</v>
       </c>
     </row>
     <row r="216">
@@ -5380,11 +5380,11 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E216" t="n">
-        <v>1</v>
+        <v>78</v>
       </c>
     </row>
     <row r="217">
@@ -5426,11 +5426,11 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E218" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
     </row>
     <row r="219">
@@ -5444,16 +5444,16 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E219" t="n">
-        <v>135</v>
+        <v>48</v>
       </c>
     </row>
     <row r="220">
@@ -5518,11 +5518,11 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E222" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
     </row>
     <row r="223">
@@ -5587,11 +5587,11 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E225" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
     </row>
     <row r="226">
@@ -6898,11 +6898,11 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
     </row>
     <row r="283">
@@ -6921,11 +6921,11 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>33</v>
+        <v>80</v>
       </c>
     </row>
     <row r="284">
@@ -6944,11 +6944,11 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
     </row>
     <row r="285">
@@ -6967,11 +6967,11 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="286">

</xml_diff>

<commit_message>
(dev): não finalizado - arquivos transitorios
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -1332,11 +1332,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>1306</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="41">
@@ -1355,11 +1355,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1105</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="42">
@@ -1373,16 +1373,16 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>791</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43">
@@ -1396,16 +1396,16 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1332</v>
+        <v>791</v>
       </c>
     </row>
     <row r="44">
@@ -1447,11 +1447,11 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
@@ -1470,11 +1470,11 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>6</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="47">
@@ -1493,11 +1493,11 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48">
@@ -1516,11 +1516,11 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
     </row>
     <row r="49">
@@ -1539,11 +1539,11 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="50">
@@ -1557,16 +1557,16 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51">
@@ -1585,11 +1585,11 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>23</v>
+        <v>41</v>
       </c>
     </row>
     <row r="52">
@@ -1603,16 +1603,16 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -1672,16 +1672,16 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>758</v>
+        <v>4380</v>
       </c>
     </row>
     <row r="56">
@@ -1718,16 +1718,16 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>4380</v>
+        <v>758</v>
       </c>
     </row>
     <row r="58">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>1</v>
+        <v>73</v>
       </c>
     </row>
     <row r="147">
@@ -3816,11 +3816,11 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149">
@@ -3839,11 +3839,11 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="150">
@@ -3862,7 +3862,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E150" t="n">
@@ -3885,11 +3885,11 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
     </row>
     <row r="152">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E152" t="n">
@@ -3931,11 +3931,11 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
     </row>
     <row r="154">
@@ -3954,11 +3954,11 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="155">
@@ -3977,11 +3977,11 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156">
@@ -4023,11 +4023,11 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="158">
@@ -4046,11 +4046,11 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="159">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E159" t="n">
@@ -4133,16 +4133,16 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>75</v>
+        <v>3286</v>
       </c>
     </row>
     <row r="163">
@@ -4184,11 +4184,11 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>528</v>
+        <v>2</v>
       </c>
     </row>
     <row r="165">
@@ -4202,16 +4202,16 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>3286</v>
+        <v>75</v>
       </c>
     </row>
     <row r="166">
@@ -4230,11 +4230,11 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>2</v>
+        <v>528</v>
       </c>
     </row>
     <row r="167">
@@ -4276,11 +4276,11 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="169">
@@ -4299,11 +4299,11 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="170">
@@ -4322,11 +4322,11 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="171">
@@ -4345,11 +4345,11 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E171" t="n">
-        <v>41</v>
+        <v>154</v>
       </c>
     </row>
     <row r="172">
@@ -4363,16 +4363,16 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>280</v>
+        <v>41</v>
       </c>
     </row>
     <row r="173">
@@ -4391,11 +4391,11 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>1</v>
+        <v>56</v>
       </c>
     </row>
     <row r="174">
@@ -4409,16 +4409,16 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E174" t="n">
-        <v>2</v>
+        <v>280</v>
       </c>
     </row>
     <row r="175">
@@ -4437,11 +4437,11 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>56</v>
+        <v>1</v>
       </c>
     </row>
     <row r="176">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E177" t="n">
-        <v>154</v>
+        <v>2</v>
       </c>
     </row>
     <row r="178">
@@ -4501,16 +4501,16 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="179">
@@ -4529,11 +4529,11 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E179" t="n">
-        <v>58</v>
+        <v>3</v>
       </c>
     </row>
     <row r="180">
@@ -4547,16 +4547,16 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E180" t="n">
-        <v>14</v>
+        <v>58</v>
       </c>
     </row>
     <row r="181">
@@ -4598,11 +4598,11 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>281</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183">
@@ -4621,11 +4621,11 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>53</v>
+        <v>281</v>
       </c>
     </row>
     <row r="184">
@@ -4667,11 +4667,11 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E185" t="n">
-        <v>1</v>
+        <v>53</v>
       </c>
     </row>
     <row r="186">
@@ -4708,16 +4708,16 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>262</v>
+        <v>391</v>
       </c>
     </row>
     <row r="188">
@@ -4782,11 +4782,11 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E190" t="n">
-        <v>217</v>
+        <v>262</v>
       </c>
     </row>
     <row r="191">
@@ -4800,16 +4800,16 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>391</v>
+        <v>217</v>
       </c>
     </row>
     <row r="192">
@@ -4828,11 +4828,11 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="193">
@@ -4846,16 +4846,16 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>64</v>
+        <v>120</v>
       </c>
     </row>
     <row r="194">
@@ -4869,16 +4869,16 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>38</v>
+        <v>64</v>
       </c>
     </row>
     <row r="195">
@@ -4966,11 +4966,11 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E198" t="n">
-        <v>1</v>
+        <v>49</v>
       </c>
     </row>
     <row r="199">
@@ -4989,11 +4989,11 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>49</v>
+        <v>284</v>
       </c>
     </row>
     <row r="200">
@@ -5012,11 +5012,11 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>284</v>
+        <v>213</v>
       </c>
     </row>
     <row r="201">
@@ -5035,11 +5035,11 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E201" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
     </row>
     <row r="202">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E202" t="n">
-        <v>213</v>
+        <v>23</v>
       </c>
     </row>
     <row r="203">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E205" t="n">
@@ -5150,11 +5150,11 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
     </row>
     <row r="207">
@@ -5173,11 +5173,11 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
     </row>
     <row r="208">
@@ -5191,16 +5191,16 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="209">
@@ -5219,11 +5219,11 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E209" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="210">
@@ -5242,11 +5242,11 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="211">
@@ -5283,16 +5283,16 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="213">
@@ -5311,11 +5311,11 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>25</v>
+        <v>11</v>
       </c>
     </row>
     <row r="214">
@@ -5380,11 +5380,11 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E216" t="n">
-        <v>78</v>
+        <v>48</v>
       </c>
     </row>
     <row r="217">
@@ -5449,11 +5449,11 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E219" t="n">
-        <v>48</v>
+        <v>78</v>
       </c>
     </row>
     <row r="220">
@@ -6185,11 +6185,11 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>2772</v>
+        <v>4187</v>
       </c>
     </row>
     <row r="252">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>4146</v>
+        <v>2772</v>
       </c>
     </row>
     <row r="253">
@@ -6231,11 +6231,11 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E253" t="n">
-        <v>4187</v>
+        <v>669</v>
       </c>
     </row>
     <row r="254">
@@ -6254,11 +6254,11 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>2</v>
+        <v>921</v>
       </c>
     </row>
     <row r="255">
@@ -6277,11 +6277,11 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>669</v>
+        <v>2</v>
       </c>
     </row>
     <row r="256">
@@ -6300,11 +6300,11 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>921</v>
+        <v>4146</v>
       </c>
     </row>
     <row r="257">
@@ -6898,11 +6898,11 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
     </row>
     <row r="283">
@@ -6921,11 +6921,11 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>80</v>
+        <v>33</v>
       </c>
     </row>
     <row r="284">
@@ -6944,11 +6944,11 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>33</v>
+        <v>3</v>
       </c>
     </row>
     <row r="285">
@@ -6967,11 +6967,11 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="286">
@@ -7128,11 +7128,11 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="293">
@@ -7151,11 +7151,11 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="294">
@@ -7174,11 +7174,11 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="295">
@@ -7197,11 +7197,11 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="296">
@@ -7243,11 +7243,11 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>897</v>
+        <v>12</v>
       </c>
     </row>
     <row r="298">
@@ -7266,11 +7266,11 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>34</v>
+        <v>897</v>
       </c>
     </row>
     <row r="299">
@@ -7289,11 +7289,11 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>287</v>
+        <v>4</v>
       </c>
     </row>
     <row r="300">
@@ -7312,11 +7312,11 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>4</v>
+        <v>34</v>
       </c>
     </row>
     <row r="301">
@@ -7335,11 +7335,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>12</v>
+        <v>287</v>
       </c>
     </row>
     <row r="302">
@@ -7772,11 +7772,11 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E320" t="n">
-        <v>44</v>
+        <v>125</v>
       </c>
     </row>
     <row r="321">
@@ -7795,11 +7795,11 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E321" t="n">
-        <v>125</v>
+        <v>300</v>
       </c>
     </row>
     <row r="322">
@@ -7818,11 +7818,11 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E322" t="n">
-        <v>300</v>
+        <v>44</v>
       </c>
     </row>
     <row r="323">
@@ -7864,11 +7864,11 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E324" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="325">
@@ -7887,11 +7887,11 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E325" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="326">
@@ -7910,11 +7910,11 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E326" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="327">
@@ -7933,11 +7933,11 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E327" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="328">

</xml_diff>

<commit_message>
chore(ploa2026): volumes ploa 3ª iteração.
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -458,11 +458,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>32</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="3">
@@ -476,16 +476,16 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>74</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="4">
@@ -504,11 +504,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>295</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5">
@@ -522,16 +522,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1251</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
@@ -550,11 +550,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2466</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7">
@@ -573,11 +573,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>26</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8">
@@ -596,11 +596,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>78</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -642,11 +642,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>429</v>
+        <v>667</v>
       </c>
     </row>
     <row r="11">
@@ -665,11 +665,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>667</v>
+        <v>429</v>
       </c>
     </row>
     <row r="12">
@@ -711,11 +711,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -734,11 +734,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -821,16 +821,16 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>110</v>
+        <v>6977</v>
       </c>
     </row>
     <row r="19">
@@ -844,16 +844,16 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>6977</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20">
@@ -1005,16 +1005,16 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="27">
@@ -1097,16 +1097,16 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31">
@@ -1120,16 +1120,16 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>60</v>
+        <v>27</v>
       </c>
     </row>
     <row r="32">
@@ -1143,16 +1143,16 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33">
@@ -1171,11 +1171,11 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34">
@@ -1194,11 +1194,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>319</v>
       </c>
     </row>
     <row r="35">
@@ -1212,16 +1212,16 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>53</v>
+        <v>222</v>
       </c>
     </row>
     <row r="36">
@@ -1235,16 +1235,16 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>222</v>
+        <v>434</v>
       </c>
     </row>
     <row r="37">
@@ -1263,11 +1263,11 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>319</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38">
@@ -1286,11 +1286,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>434</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
@@ -1309,11 +1309,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>5</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="40">
@@ -1332,11 +1332,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>778</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="41">
@@ -1350,16 +1350,16 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>483</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="42">
@@ -1378,11 +1378,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1365</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43">
@@ -1401,11 +1401,11 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1086</v>
+        <v>778</v>
       </c>
     </row>
     <row r="44">
@@ -1419,16 +1419,16 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>1483</v>
+        <v>483</v>
       </c>
     </row>
     <row r="45">
@@ -1447,11 +1447,11 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="46">
@@ -1470,11 +1470,11 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>23</v>
+        <v>41</v>
       </c>
     </row>
     <row r="47">
@@ -1488,16 +1488,16 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48">
@@ -1516,11 +1516,11 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -1539,11 +1539,11 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
     </row>
     <row r="50">
@@ -1557,16 +1557,16 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51">
@@ -1585,11 +1585,11 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>5</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="52">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>767</v>
+        <v>570</v>
       </c>
     </row>
     <row r="53">
@@ -1626,16 +1626,16 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>4293</v>
+        <v>767</v>
       </c>
     </row>
     <row r="54">
@@ -1654,11 +1654,11 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>570</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55">
@@ -1672,16 +1672,16 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>1506</v>
+        <v>4293</v>
       </c>
     </row>
     <row r="56">
@@ -1700,11 +1700,11 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>8</v>
+        <v>133</v>
       </c>
     </row>
     <row r="57">
@@ -1718,16 +1718,16 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>409</v>
+        <v>46</v>
       </c>
     </row>
     <row r="58">
@@ -1746,11 +1746,11 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>133</v>
+        <v>8</v>
       </c>
     </row>
     <row r="59">
@@ -1764,16 +1764,16 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>46</v>
+        <v>409</v>
       </c>
     </row>
     <row r="60">
@@ -1792,11 +1792,11 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>2</v>
+        <v>45</v>
       </c>
     </row>
     <row r="61">
@@ -1810,16 +1810,16 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>108</v>
+        <v>481</v>
       </c>
     </row>
     <row r="62">
@@ -1833,16 +1833,16 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>481</v>
+        <v>41</v>
       </c>
     </row>
     <row r="63">
@@ -1861,11 +1861,11 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>45</v>
+        <v>108</v>
       </c>
     </row>
     <row r="64">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65">
@@ -1907,11 +1907,11 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>3</v>
+        <v>190</v>
       </c>
     </row>
     <row r="66">
@@ -1930,11 +1930,11 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>237</v>
+        <v>2339</v>
       </c>
     </row>
     <row r="67">
@@ -1953,11 +1953,11 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>1</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="68">
@@ -1976,11 +1976,11 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>190</v>
+        <v>3764</v>
       </c>
     </row>
     <row r="69">
@@ -1994,16 +1994,16 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>39337</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -2017,16 +2017,16 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>1793</v>
+        <v>470</v>
       </c>
     </row>
     <row r="71">
@@ -2040,16 +2040,16 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>3764</v>
+        <v>39337</v>
       </c>
     </row>
     <row r="72">
@@ -2068,11 +2068,11 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>33828</v>
+        <v>3</v>
       </c>
     </row>
     <row r="73">
@@ -2086,16 +2086,16 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>470</v>
+        <v>237</v>
       </c>
     </row>
     <row r="74">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>2339</v>
+        <v>33828</v>
       </c>
     </row>
     <row r="75">
@@ -2137,11 +2137,11 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>6</v>
+        <v>14014</v>
       </c>
     </row>
     <row r="76">
@@ -2160,11 +2160,11 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>4144</v>
+        <v>158968</v>
       </c>
     </row>
     <row r="77">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>23323</v>
+        <v>37607</v>
       </c>
     </row>
     <row r="78">
@@ -2201,16 +2201,16 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>176055</v>
+        <v>23323</v>
       </c>
     </row>
     <row r="79">
@@ -2229,11 +2229,11 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>158968</v>
+        <v>6</v>
       </c>
     </row>
     <row r="80">
@@ -2252,11 +2252,11 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>37607</v>
+        <v>4144</v>
       </c>
     </row>
     <row r="81">
@@ -2270,16 +2270,16 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>14014</v>
+        <v>176055</v>
       </c>
     </row>
     <row r="82">
@@ -2298,11 +2298,11 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>4</v>
+        <v>80</v>
       </c>
     </row>
     <row r="83">
@@ -2321,11 +2321,11 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>157</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84">
@@ -2339,16 +2339,16 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>276</v>
+        <v>15</v>
       </c>
     </row>
     <row r="85">
@@ -2367,11 +2367,11 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>80</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86">
@@ -2390,11 +2390,11 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>3</v>
+        <v>157</v>
       </c>
     </row>
     <row r="87">
@@ -2408,16 +2408,16 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>15</v>
+        <v>276</v>
       </c>
     </row>
     <row r="88">
@@ -2436,11 +2436,11 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>7</v>
+        <v>124</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>44</v>
+        <v>89</v>
       </c>
     </row>
     <row r="90">
@@ -2477,16 +2477,16 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>74</v>
+        <v>44</v>
       </c>
     </row>
     <row r="91">
@@ -2505,11 +2505,11 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>89</v>
+        <v>7</v>
       </c>
     </row>
     <row r="92">
@@ -2523,16 +2523,16 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>124</v>
+        <v>74</v>
       </c>
     </row>
     <row r="93">
@@ -2546,16 +2546,16 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="94">
@@ -2574,11 +2574,11 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>83</v>
+        <v>10</v>
       </c>
     </row>
     <row r="95">
@@ -2592,16 +2592,16 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>21</v>
+        <v>333</v>
       </c>
     </row>
     <row r="96">
@@ -2620,11 +2620,11 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>333</v>
+        <v>75</v>
       </c>
     </row>
     <row r="97">
@@ -2643,11 +2643,11 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>75</v>
+        <v>83</v>
       </c>
     </row>
     <row r="98">
@@ -2666,11 +2666,11 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>2</v>
+        <v>724</v>
       </c>
     </row>
     <row r="99">
@@ -2689,11 +2689,11 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>22</v>
+        <v>5145</v>
       </c>
     </row>
     <row r="100">
@@ -2707,16 +2707,16 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>3219</v>
+        <v>22</v>
       </c>
     </row>
     <row r="101">
@@ -2735,11 +2735,11 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>5145</v>
+        <v>2</v>
       </c>
     </row>
     <row r="102">
@@ -2753,16 +2753,16 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>724</v>
+        <v>3219</v>
       </c>
     </row>
     <row r="103">
@@ -2781,11 +2781,11 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E103" t="n">
-        <v>5</v>
+        <v>69</v>
       </c>
     </row>
     <row r="104">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>114</v>
+        <v>6</v>
       </c>
     </row>
     <row r="105">
@@ -2850,11 +2850,11 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>69</v>
+        <v>5</v>
       </c>
     </row>
     <row r="107">
@@ -2873,11 +2873,11 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>6</v>
+        <v>114</v>
       </c>
     </row>
     <row r="108">
@@ -2919,11 +2919,11 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="110">
@@ -2942,11 +2942,11 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>285</v>
+        <v>17855</v>
       </c>
     </row>
     <row r="111">
@@ -2960,16 +2960,16 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>3</v>
+        <v>830</v>
       </c>
     </row>
     <row r="112">
@@ -2988,11 +2988,11 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>17855</v>
+        <v>9</v>
       </c>
     </row>
     <row r="113">
@@ -3052,16 +3052,16 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>830</v>
+        <v>285</v>
       </c>
     </row>
     <row r="116">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>287</v>
+        <v>147</v>
       </c>
     </row>
     <row r="117">
@@ -3126,11 +3126,11 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>142</v>
+        <v>287</v>
       </c>
     </row>
     <row r="119">
@@ -3144,16 +3144,16 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>1151</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120">
@@ -3172,11 +3172,11 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>11</v>
+        <v>142</v>
       </c>
     </row>
     <row r="121">
@@ -3190,16 +3190,16 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>2</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="122">
@@ -3218,11 +3218,11 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>147</v>
+        <v>11</v>
       </c>
     </row>
     <row r="123">
@@ -3241,11 +3241,11 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>262</v>
+        <v>46</v>
       </c>
     </row>
     <row r="124">
@@ -3264,11 +3264,11 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>63</v>
+        <v>262</v>
       </c>
     </row>
     <row r="125">
@@ -3282,16 +3282,16 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>1073</v>
+        <v>63</v>
       </c>
     </row>
     <row r="126">
@@ -3305,16 +3305,16 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E126" t="n">
-        <v>46</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="127">
@@ -3351,16 +3351,16 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E128" t="n">
-        <v>1589</v>
+        <v>624</v>
       </c>
     </row>
     <row r="129">
@@ -3374,16 +3374,16 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>751</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="130">
@@ -3402,11 +3402,11 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>624</v>
+        <v>751</v>
       </c>
     </row>
     <row r="131">
@@ -3494,11 +3494,11 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>19</v>
+        <v>43</v>
       </c>
     </row>
     <row r="135">
@@ -3535,16 +3535,16 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E136" t="n">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="137">
@@ -3581,16 +3581,16 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E138" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
     </row>
     <row r="139">
@@ -3632,11 +3632,11 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E140" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141">
@@ -3650,16 +3650,16 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E141" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="142">
@@ -3673,16 +3673,16 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E142" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="143">
@@ -3701,11 +3701,11 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E143" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="144">
@@ -3724,11 +3724,11 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
     </row>
     <row r="145">
@@ -3747,11 +3747,11 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="146">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147">
@@ -3793,11 +3793,11 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="148">
@@ -3816,11 +3816,11 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
     </row>
     <row r="149">
@@ -3862,11 +3862,11 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E150" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="151">
@@ -3885,11 +3885,11 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="152">
@@ -3931,11 +3931,11 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
     </row>
     <row r="154">
@@ -3954,11 +3954,11 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="155">
@@ -3977,11 +3977,11 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
     </row>
     <row r="156">
@@ -4000,11 +4000,11 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E156" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="157">
@@ -4023,11 +4023,11 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>75</v>
+        <v>2</v>
       </c>
     </row>
     <row r="158">
@@ -4041,16 +4041,16 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>2</v>
+        <v>3346</v>
       </c>
     </row>
     <row r="159">
@@ -4092,11 +4092,11 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E160" t="n">
-        <v>807</v>
+        <v>916</v>
       </c>
     </row>
     <row r="161">
@@ -4110,16 +4110,16 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E161" t="n">
-        <v>3346</v>
+        <v>807</v>
       </c>
     </row>
     <row r="162">
@@ -4138,11 +4138,11 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>916</v>
+        <v>75</v>
       </c>
     </row>
     <row r="163">
@@ -4161,11 +4161,11 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="164">
@@ -4179,16 +4179,16 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
     </row>
     <row r="165">
@@ -4202,16 +4202,16 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="166">
@@ -4230,11 +4230,11 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="167">
@@ -4248,16 +4248,16 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E167" t="n">
-        <v>43</v>
+        <v>281</v>
       </c>
     </row>
     <row r="168">
@@ -4271,16 +4271,16 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>281</v>
+        <v>1</v>
       </c>
     </row>
     <row r="169">
@@ -4299,11 +4299,11 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>148</v>
+        <v>2</v>
       </c>
     </row>
     <row r="170">
@@ -4368,11 +4368,11 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>1</v>
+        <v>43</v>
       </c>
     </row>
     <row r="173">
@@ -4391,11 +4391,11 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>2</v>
+        <v>148</v>
       </c>
     </row>
     <row r="174">
@@ -4409,16 +4409,16 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E174" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="175">
@@ -4437,11 +4437,11 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>62</v>
+        <v>24</v>
       </c>
     </row>
     <row r="176">
@@ -4455,16 +4455,16 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E176" t="n">
-        <v>13</v>
+        <v>62</v>
       </c>
     </row>
     <row r="177">
@@ -4501,16 +4501,16 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>296</v>
+        <v>95</v>
       </c>
     </row>
     <row r="179">
@@ -4524,16 +4524,16 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E179" t="n">
-        <v>95</v>
+        <v>53</v>
       </c>
     </row>
     <row r="180">
@@ -4552,11 +4552,11 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E180" t="n">
-        <v>53</v>
+        <v>78</v>
       </c>
     </row>
     <row r="181">
@@ -4575,11 +4575,11 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
@@ -4598,11 +4598,11 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>1</v>
+        <v>296</v>
       </c>
     </row>
     <row r="183">
@@ -4621,11 +4621,11 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>217</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184">
@@ -4644,11 +4644,11 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E184" t="n">
-        <v>266</v>
+        <v>262</v>
       </c>
     </row>
     <row r="185">
@@ -4667,11 +4667,11 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E185" t="n">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="186">
@@ -4685,16 +4685,16 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E186" t="n">
-        <v>391</v>
+        <v>217</v>
       </c>
     </row>
     <row r="187">
@@ -4708,16 +4708,16 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>1</v>
+        <v>391</v>
       </c>
     </row>
     <row r="188">
@@ -4736,11 +4736,11 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>4</v>
+        <v>109</v>
       </c>
     </row>
     <row r="189">
@@ -4759,11 +4759,11 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="190">
@@ -4782,11 +4782,11 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E190" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
     </row>
     <row r="191">
@@ -4800,16 +4800,16 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>109</v>
+        <v>60</v>
       </c>
     </row>
     <row r="192">
@@ -4823,16 +4823,16 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
     </row>
     <row r="193">
@@ -4846,16 +4846,16 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>50</v>
+        <v>205</v>
       </c>
     </row>
     <row r="194">
@@ -4869,16 +4869,16 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>22</v>
+        <v>50</v>
       </c>
     </row>
     <row r="195">
@@ -4897,11 +4897,11 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E195" t="n">
-        <v>4</v>
+        <v>332</v>
       </c>
     </row>
     <row r="196">
@@ -4920,11 +4920,11 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="197">
@@ -4943,11 +4943,11 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
     </row>
     <row r="198">
@@ -4966,11 +4966,11 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E198" t="n">
-        <v>205</v>
+        <v>22</v>
       </c>
     </row>
     <row r="199">
@@ -4989,11 +4989,11 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>332</v>
+        <v>4</v>
       </c>
     </row>
     <row r="200">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E200" t="n">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E203" t="n">
@@ -5104,11 +5104,11 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E204" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="205">
@@ -5122,16 +5122,16 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="206">
@@ -5145,16 +5145,16 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="207">
@@ -5173,11 +5173,11 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="208">
@@ -5196,11 +5196,11 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
     </row>
     <row r="209">
@@ -5219,11 +5219,11 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E209" t="n">
-        <v>46</v>
+        <v>78</v>
       </c>
     </row>
     <row r="210">
@@ -5260,16 +5260,16 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>136</v>
+        <v>55</v>
       </c>
     </row>
     <row r="212">
@@ -5288,11 +5288,11 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
     </row>
     <row r="213">
@@ -5306,16 +5306,16 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>78</v>
+        <v>136</v>
       </c>
     </row>
     <row r="214">
@@ -5334,11 +5334,11 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E214" t="n">
-        <v>1</v>
+        <v>46</v>
       </c>
     </row>
     <row r="215">
@@ -7565,11 +7565,11 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E311" t="n">
-        <v>887</v>
+        <v>5</v>
       </c>
     </row>
     <row r="312">
@@ -7583,16 +7583,16 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E312" t="n">
-        <v>93</v>
+        <v>448</v>
       </c>
     </row>
     <row r="313">
@@ -7611,11 +7611,11 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E313" t="n">
-        <v>40</v>
+        <v>887</v>
       </c>
     </row>
     <row r="314">
@@ -7634,11 +7634,11 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E314" t="n">
-        <v>328</v>
+        <v>40</v>
       </c>
     </row>
     <row r="315">
@@ -7657,11 +7657,11 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E315" t="n">
-        <v>448</v>
+        <v>328</v>
       </c>
     </row>
     <row r="316">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>3041 - EMATER</t>
+          <t>3051 - EPAMIG</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -7680,11 +7680,11 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E316" t="n">
-        <v>5</v>
+        <v>291</v>
       </c>
     </row>
     <row r="317">
@@ -7703,11 +7703,11 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E317" t="n">
-        <v>44</v>
+        <v>189</v>
       </c>
     </row>
     <row r="318">
@@ -7726,11 +7726,11 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E318" t="n">
-        <v>189</v>
+        <v>44</v>
       </c>
     </row>
     <row r="319">
@@ -7762,7 +7762,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>3051 - EPAMIG</t>
+          <t>3151 - EMC</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -7772,11 +7772,11 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E320" t="n">
-        <v>291</v>
+        <v>30</v>
       </c>
     </row>
     <row r="321">
@@ -7795,11 +7795,11 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E321" t="n">
-        <v>16</v>
+        <v>56</v>
       </c>
     </row>
     <row r="322">
@@ -7818,11 +7818,11 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E322" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="323">
@@ -7841,11 +7841,11 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E323" t="n">
-        <v>56</v>
+        <v>7</v>
       </c>
     </row>
     <row r="324">
@@ -7864,11 +7864,11 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E324" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
     </row>
     <row r="325">
@@ -7877,7 +7877,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>3151 - EMC</t>
+          <t>4291 - FES</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -7887,11 +7887,11 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E325" t="n">
-        <v>37</v>
+        <v>10</v>
       </c>
     </row>
     <row r="326">
@@ -7910,11 +7910,11 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E326" t="n">
-        <v>10</v>
+        <v>84</v>
       </c>
     </row>
     <row r="327">
@@ -7933,11 +7933,11 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E327" t="n">
-        <v>84</v>
+        <v>250</v>
       </c>
     </row>
     <row r="328">
@@ -7951,16 +7951,16 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E328" t="n">
-        <v>250</v>
+        <v>8614</v>
       </c>
     </row>
     <row r="329">
@@ -7974,16 +7974,16 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E329" t="n">
-        <v>8614</v>
+        <v>949</v>
       </c>
     </row>
     <row r="330">
@@ -8002,11 +8002,11 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E330" t="n">
-        <v>949</v>
+        <v>449</v>
       </c>
     </row>
     <row r="331">
@@ -8025,33 +8025,10 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E331" t="n">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B332" t="inlineStr">
-        <is>
-          <t>4291 - FES</t>
-        </is>
-      </c>
-      <c r="C332" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="D332" t="inlineStr">
-        <is>
-          <t>ESPECIALIZADA</t>
-        </is>
-      </c>
-      <c r="E332" t="n">
         <v>1925</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: Demonstrativos pós emendas, 1ª iteração.
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -458,11 +458,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2466</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -476,16 +476,16 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1251</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4">
@@ -504,11 +504,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>74</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5">
@@ -522,16 +522,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>32</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="6">
@@ -550,11 +550,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>78</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="7">
@@ -573,11 +573,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>295</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8">
@@ -596,11 +596,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>26</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9">
@@ -642,11 +642,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>667</v>
+        <v>429</v>
       </c>
     </row>
     <row r="11">
@@ -665,11 +665,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>429</v>
+        <v>667</v>
       </c>
     </row>
     <row r="12">
@@ -711,11 +711,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -734,11 +734,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
@@ -821,16 +821,16 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>6977</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19">
@@ -844,16 +844,16 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>110</v>
+        <v>6977</v>
       </c>
     </row>
     <row r="20">
@@ -1005,16 +1005,16 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27">
@@ -1097,16 +1097,16 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31">
@@ -1120,16 +1120,16 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32">
@@ -1143,16 +1143,16 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33">
@@ -1171,11 +1171,11 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34">
@@ -1194,11 +1194,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>319</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -1212,16 +1212,16 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>222</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36">
@@ -1235,16 +1235,16 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>434</v>
+        <v>222</v>
       </c>
     </row>
     <row r="37">
@@ -1263,11 +1263,11 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>53</v>
+        <v>319</v>
       </c>
     </row>
     <row r="38">
@@ -1286,11 +1286,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>434</v>
       </c>
     </row>
     <row r="39">
@@ -1309,11 +1309,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1365</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
@@ -1332,11 +1332,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>1086</v>
+        <v>778</v>
       </c>
     </row>
     <row r="41">
@@ -1350,16 +1350,16 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1483</v>
+        <v>483</v>
       </c>
     </row>
     <row r="42">
@@ -1378,11 +1378,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>5</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="43">
@@ -1401,11 +1401,11 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>778</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="44">
@@ -1419,16 +1419,16 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>483</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="45">
@@ -1447,11 +1447,11 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -1470,11 +1470,11 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
     </row>
     <row r="47">
@@ -1488,16 +1488,16 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -1516,11 +1516,11 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="49">
@@ -1539,11 +1539,11 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>23</v>
+        <v>41</v>
       </c>
     </row>
     <row r="50">
@@ -1557,16 +1557,16 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="51">
@@ -1585,11 +1585,11 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>1506</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>570</v>
+        <v>767</v>
       </c>
     </row>
     <row r="53">
@@ -1626,16 +1626,16 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>767</v>
+        <v>4293</v>
       </c>
     </row>
     <row r="54">
@@ -1654,11 +1654,11 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>5</v>
+        <v>570</v>
       </c>
     </row>
     <row r="55">
@@ -1672,16 +1672,16 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>4293</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="56">
@@ -1700,11 +1700,11 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>133</v>
+        <v>8</v>
       </c>
     </row>
     <row r="57">
@@ -1718,16 +1718,16 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>46</v>
+        <v>409</v>
       </c>
     </row>
     <row r="58">
@@ -1746,11 +1746,11 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>8</v>
+        <v>133</v>
       </c>
     </row>
     <row r="59">
@@ -1764,16 +1764,16 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>409</v>
+        <v>46</v>
       </c>
     </row>
     <row r="60">
@@ -1792,11 +1792,11 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>45</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
@@ -1810,16 +1810,16 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>481</v>
+        <v>108</v>
       </c>
     </row>
     <row r="62">
@@ -1833,16 +1833,16 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>41</v>
+        <v>481</v>
       </c>
     </row>
     <row r="63">
@@ -1861,11 +1861,11 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>108</v>
+        <v>45</v>
       </c>
     </row>
     <row r="64">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>41</v>
       </c>
     </row>
     <row r="65">
@@ -1907,11 +1907,11 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>190</v>
+        <v>3</v>
       </c>
     </row>
     <row r="66">
@@ -1930,11 +1930,11 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>2339</v>
+        <v>237</v>
       </c>
     </row>
     <row r="67">
@@ -1953,11 +1953,11 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>1793</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
@@ -1976,11 +1976,11 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>3764</v>
+        <v>190</v>
       </c>
     </row>
     <row r="69">
@@ -1994,16 +1994,16 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>1</v>
+        <v>39337</v>
       </c>
     </row>
     <row r="70">
@@ -2017,16 +2017,16 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>470</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="71">
@@ -2040,16 +2040,16 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>39337</v>
+        <v>3764</v>
       </c>
     </row>
     <row r="72">
@@ -2068,11 +2068,11 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>3</v>
+        <v>33828</v>
       </c>
     </row>
     <row r="73">
@@ -2086,16 +2086,16 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>237</v>
+        <v>470</v>
       </c>
     </row>
     <row r="74">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>33828</v>
+        <v>2339</v>
       </c>
     </row>
     <row r="75">
@@ -2137,11 +2137,11 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>14014</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76">
@@ -2160,11 +2160,11 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>158968</v>
+        <v>4144</v>
       </c>
     </row>
     <row r="77">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>37607</v>
+        <v>23323</v>
       </c>
     </row>
     <row r="78">
@@ -2201,16 +2201,16 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>23323</v>
+        <v>176055</v>
       </c>
     </row>
     <row r="79">
@@ -2229,11 +2229,11 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>6</v>
+        <v>158968</v>
       </c>
     </row>
     <row r="80">
@@ -2252,11 +2252,11 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>4144</v>
+        <v>37607</v>
       </c>
     </row>
     <row r="81">
@@ -2270,16 +2270,16 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>176055</v>
+        <v>14014</v>
       </c>
     </row>
     <row r="82">
@@ -2298,11 +2298,11 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>80</v>
+        <v>4</v>
       </c>
     </row>
     <row r="83">
@@ -2321,11 +2321,11 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>3</v>
+        <v>157</v>
       </c>
     </row>
     <row r="84">
@@ -2339,16 +2339,16 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>15</v>
+        <v>276</v>
       </c>
     </row>
     <row r="85">
@@ -2367,11 +2367,11 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>4</v>
+        <v>80</v>
       </c>
     </row>
     <row r="86">
@@ -2390,11 +2390,11 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>157</v>
+        <v>3</v>
       </c>
     </row>
     <row r="87">
@@ -2408,16 +2408,16 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>276</v>
+        <v>15</v>
       </c>
     </row>
     <row r="88">
@@ -2436,11 +2436,11 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>124</v>
+        <v>7</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>89</v>
+        <v>44</v>
       </c>
     </row>
     <row r="90">
@@ -2477,16 +2477,16 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>44</v>
+        <v>74</v>
       </c>
     </row>
     <row r="91">
@@ -2505,11 +2505,11 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>7</v>
+        <v>89</v>
       </c>
     </row>
     <row r="92">
@@ -2523,16 +2523,16 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>74</v>
+        <v>124</v>
       </c>
     </row>
     <row r="93">
@@ -2546,16 +2546,16 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="94">
@@ -2574,11 +2574,11 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>10</v>
+        <v>83</v>
       </c>
     </row>
     <row r="95">
@@ -2592,16 +2592,16 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>333</v>
+        <v>21</v>
       </c>
     </row>
     <row r="96">
@@ -2620,11 +2620,11 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>75</v>
+        <v>333</v>
       </c>
     </row>
     <row r="97">
@@ -2643,11 +2643,11 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="98">
@@ -2666,11 +2666,11 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>724</v>
+        <v>2</v>
       </c>
     </row>
     <row r="99">
@@ -2689,11 +2689,11 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>5145</v>
+        <v>22</v>
       </c>
     </row>
     <row r="100">
@@ -2707,16 +2707,16 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>22</v>
+        <v>3219</v>
       </c>
     </row>
     <row r="101">
@@ -2735,11 +2735,11 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>2</v>
+        <v>5145</v>
       </c>
     </row>
     <row r="102">
@@ -2753,16 +2753,16 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>3219</v>
+        <v>724</v>
       </c>
     </row>
     <row r="103">
@@ -2781,11 +2781,11 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E103" t="n">
-        <v>69</v>
+        <v>5</v>
       </c>
     </row>
     <row r="104">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>6</v>
+        <v>114</v>
       </c>
     </row>
     <row r="105">
@@ -2850,11 +2850,11 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>5</v>
+        <v>69</v>
       </c>
     </row>
     <row r="107">
@@ -2873,11 +2873,11 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>114</v>
+        <v>6</v>
       </c>
     </row>
     <row r="108">
@@ -2919,11 +2919,11 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="110">
@@ -2942,11 +2942,11 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>17855</v>
+        <v>285</v>
       </c>
     </row>
     <row r="111">
@@ -2960,16 +2960,16 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>830</v>
+        <v>3</v>
       </c>
     </row>
     <row r="112">
@@ -2988,11 +2988,11 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>9</v>
+        <v>17855</v>
       </c>
     </row>
     <row r="113">
@@ -3052,16 +3052,16 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>285</v>
+        <v>830</v>
       </c>
     </row>
     <row r="116">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>147</v>
+        <v>287</v>
       </c>
     </row>
     <row r="117">
@@ -3126,11 +3126,11 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>287</v>
+        <v>142</v>
       </c>
     </row>
     <row r="119">
@@ -3144,16 +3144,16 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>2</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="120">
@@ -3172,11 +3172,11 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>142</v>
+        <v>11</v>
       </c>
     </row>
     <row r="121">
@@ -3190,16 +3190,16 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>1151</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122">
@@ -3218,11 +3218,11 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>11</v>
+        <v>147</v>
       </c>
     </row>
     <row r="123">
@@ -3241,11 +3241,11 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>46</v>
+        <v>262</v>
       </c>
     </row>
     <row r="124">
@@ -3264,11 +3264,11 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>262</v>
+        <v>63</v>
       </c>
     </row>
     <row r="125">
@@ -3282,16 +3282,16 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>63</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="126">
@@ -3305,16 +3305,16 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E126" t="n">
-        <v>1073</v>
+        <v>46</v>
       </c>
     </row>
     <row r="127">
@@ -3351,16 +3351,16 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E128" t="n">
-        <v>624</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="129">
@@ -3374,16 +3374,16 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>1589</v>
+        <v>751</v>
       </c>
     </row>
     <row r="130">
@@ -3402,11 +3402,11 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>751</v>
+        <v>624</v>
       </c>
     </row>
     <row r="131">
@@ -3494,11 +3494,11 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>43</v>
+        <v>19</v>
       </c>
     </row>
     <row r="135">
@@ -3535,16 +3535,16 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E136" t="n">
-        <v>34</v>
+        <v>43</v>
       </c>
     </row>
     <row r="137">
@@ -3581,16 +3581,16 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E138" t="n">
-        <v>19</v>
+        <v>34</v>
       </c>
     </row>
     <row r="139">
@@ -3632,11 +3632,11 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E140" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="141">
@@ -3650,16 +3650,16 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E141" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142">
@@ -3673,16 +3673,16 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E142" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="143">
@@ -3701,11 +3701,11 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E143" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="144">
@@ -3724,11 +3724,11 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145">
@@ -3747,11 +3747,11 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="146">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="147">
@@ -3793,11 +3793,11 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="148">
@@ -3816,11 +3816,11 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
     </row>
     <row r="149">
@@ -3862,11 +3862,11 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E150" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="151">
@@ -3885,11 +3885,11 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="152">
@@ -3931,11 +3931,11 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
     </row>
     <row r="154">
@@ -3954,11 +3954,11 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="155">
@@ -3977,11 +3977,11 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
     </row>
     <row r="156">
@@ -4000,11 +4000,11 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E156" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="157">
@@ -4023,11 +4023,11 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>2</v>
+        <v>75</v>
       </c>
     </row>
     <row r="158">
@@ -4041,16 +4041,16 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>3346</v>
+        <v>2</v>
       </c>
     </row>
     <row r="159">
@@ -4092,11 +4092,11 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E160" t="n">
-        <v>916</v>
+        <v>807</v>
       </c>
     </row>
     <row r="161">
@@ -4110,16 +4110,16 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E161" t="n">
-        <v>807</v>
+        <v>3346</v>
       </c>
     </row>
     <row r="162">
@@ -4138,11 +4138,11 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>75</v>
+        <v>916</v>
       </c>
     </row>
     <row r="163">
@@ -4161,11 +4161,11 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="164">
@@ -4179,16 +4179,16 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="165">
@@ -4202,16 +4202,16 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
     </row>
     <row r="166">
@@ -4230,11 +4230,11 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="167">
@@ -4248,16 +4248,16 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E167" t="n">
-        <v>281</v>
+        <v>43</v>
       </c>
     </row>
     <row r="168">
@@ -4271,16 +4271,16 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>1</v>
+        <v>281</v>
       </c>
     </row>
     <row r="169">
@@ -4299,11 +4299,11 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>2</v>
+        <v>148</v>
       </c>
     </row>
     <row r="170">
@@ -4368,11 +4368,11 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173">
@@ -4391,11 +4391,11 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>148</v>
+        <v>2</v>
       </c>
     </row>
     <row r="174">
@@ -4409,16 +4409,16 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E174" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="175">
@@ -4437,11 +4437,11 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>24</v>
+        <v>62</v>
       </c>
     </row>
     <row r="176">
@@ -4455,16 +4455,16 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E176" t="n">
-        <v>62</v>
+        <v>13</v>
       </c>
     </row>
     <row r="177">
@@ -4501,16 +4501,16 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>95</v>
+        <v>296</v>
       </c>
     </row>
     <row r="179">
@@ -4524,16 +4524,16 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E179" t="n">
-        <v>53</v>
+        <v>95</v>
       </c>
     </row>
     <row r="180">
@@ -4552,11 +4552,11 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E180" t="n">
-        <v>78</v>
+        <v>53</v>
       </c>
     </row>
     <row r="181">
@@ -4575,11 +4575,11 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>1</v>
+        <v>78</v>
       </c>
     </row>
     <row r="182">
@@ -4598,11 +4598,11 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>296</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183">
@@ -4621,11 +4621,11 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>1</v>
+        <v>217</v>
       </c>
     </row>
     <row r="184">
@@ -4644,11 +4644,11 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E184" t="n">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="185">
@@ -4667,11 +4667,11 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E185" t="n">
-        <v>266</v>
+        <v>262</v>
       </c>
     </row>
     <row r="186">
@@ -4685,16 +4685,16 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E186" t="n">
-        <v>217</v>
+        <v>391</v>
       </c>
     </row>
     <row r="187">
@@ -4708,16 +4708,16 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>391</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188">
@@ -4736,11 +4736,11 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>109</v>
+        <v>4</v>
       </c>
     </row>
     <row r="189">
@@ -4759,11 +4759,11 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="190">
@@ -4782,11 +4782,11 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E190" t="n">
-        <v>4</v>
+        <v>38</v>
       </c>
     </row>
     <row r="191">
@@ -4800,16 +4800,16 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>60</v>
+        <v>109</v>
       </c>
     </row>
     <row r="192">
@@ -4823,16 +4823,16 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
     </row>
     <row r="193">
@@ -4846,16 +4846,16 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>205</v>
+        <v>50</v>
       </c>
     </row>
     <row r="194">
@@ -4869,16 +4869,16 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
     </row>
     <row r="195">
@@ -4897,11 +4897,11 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E195" t="n">
-        <v>332</v>
+        <v>4</v>
       </c>
     </row>
     <row r="196">
@@ -4920,11 +4920,11 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
     </row>
     <row r="197">
@@ -4943,11 +4943,11 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="198">
@@ -4966,11 +4966,11 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E198" t="n">
-        <v>22</v>
+        <v>205</v>
       </c>
     </row>
     <row r="199">
@@ -4989,11 +4989,11 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>4</v>
+        <v>332</v>
       </c>
     </row>
     <row r="200">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E200" t="n">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E203" t="n">
@@ -5104,11 +5104,11 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E204" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="205">
@@ -5122,16 +5122,16 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="206">
@@ -5145,16 +5145,16 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="207">
@@ -5173,11 +5173,11 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="208">
@@ -5196,11 +5196,11 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
     </row>
     <row r="209">
@@ -5219,11 +5219,11 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E209" t="n">
-        <v>78</v>
+        <v>46</v>
       </c>
     </row>
     <row r="210">
@@ -5260,16 +5260,16 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>55</v>
+        <v>136</v>
       </c>
     </row>
     <row r="212">
@@ -5288,11 +5288,11 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
     </row>
     <row r="213">
@@ -5306,16 +5306,16 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>136</v>
+        <v>78</v>
       </c>
     </row>
     <row r="214">
@@ -5334,11 +5334,11 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E214" t="n">
-        <v>46</v>
+        <v>1</v>
       </c>
     </row>
     <row r="215">

</xml_diff>

<commit_message>
atualiza volumes loa com ppo - 08092026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -7141,7 +7141,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -7155,7 +7155,7 @@
         </is>
       </c>
       <c r="E293" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="294">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -7178,7 +7178,7 @@
         </is>
       </c>
       <c r="E294" t="n">
-        <v>158</v>
+        <v>3781</v>
       </c>
     </row>
     <row r="295">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -7201,7 +7201,7 @@
         </is>
       </c>
       <c r="E295" t="n">
-        <v>56</v>
+        <v>107</v>
       </c>
     </row>
     <row r="296">
@@ -7210,7 +7210,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7224,7 +7224,7 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>38</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="297">
@@ -7233,7 +7233,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -7243,11 +7243,11 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>1</v>
+        <v>8398</v>
       </c>
     </row>
     <row r="298">
@@ -7256,21 +7256,21 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>273</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="299">
@@ -7279,21 +7279,21 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>7</v>
+        <v>6858</v>
       </c>
     </row>
     <row r="300">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -7312,11 +7312,11 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="301">
@@ -7325,7 +7325,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -7335,11 +7335,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>22</v>
+        <v>158</v>
       </c>
     </row>
     <row r="302">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="303">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -7381,11 +7381,11 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>282</v>
+        <v>38</v>
       </c>
     </row>
     <row r="304">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -7404,11 +7404,11 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>205</v>
+        <v>1</v>
       </c>
     </row>
     <row r="305">
@@ -7417,7 +7417,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -7431,7 +7431,7 @@
         </is>
       </c>
       <c r="E305" t="n">
-        <v>53</v>
+        <v>273</v>
       </c>
     </row>
     <row r="306">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -7454,7 +7454,7 @@
         </is>
       </c>
       <c r="E306" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="307">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -7477,7 +7477,7 @@
         </is>
       </c>
       <c r="E307" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="308">
@@ -7486,7 +7486,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -7496,11 +7496,11 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E308" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="309">
@@ -7509,7 +7509,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -7519,11 +7519,11 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>17</v>
+        <v>48</v>
       </c>
     </row>
     <row r="310">
@@ -7532,7 +7532,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -7542,11 +7542,11 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>1</v>
+        <v>282</v>
       </c>
     </row>
     <row r="311">
@@ -7555,7 +7555,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -7565,11 +7565,11 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E311" t="n">
-        <v>24</v>
+        <v>205</v>
       </c>
     </row>
     <row r="312">
@@ -7578,21 +7578,21 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E312" t="n">
-        <v>16</v>
+        <v>53</v>
       </c>
     </row>
     <row r="313">
@@ -7601,7 +7601,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -7611,11 +7611,11 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E313" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
     </row>
     <row r="314">
@@ -7624,7 +7624,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -7634,11 +7634,11 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E314" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
     </row>
     <row r="315">
@@ -7647,21 +7647,21 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E315" t="n">
-        <v>32</v>
+        <v>17</v>
       </c>
     </row>
     <row r="316">
@@ -7670,21 +7670,21 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>1941 - EGE-SEPLAG</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E316" t="n">
-        <v>1703</v>
+        <v>17</v>
       </c>
     </row>
     <row r="317">
@@ -7693,7 +7693,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -7707,7 +7707,7 @@
         </is>
       </c>
       <c r="E317" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="318">
@@ -7716,7 +7716,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -7730,7 +7730,7 @@
         </is>
       </c>
       <c r="E318" t="n">
-        <v>4125</v>
+        <v>24</v>
       </c>
     </row>
     <row r="319">
@@ -7739,7 +7739,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -7753,7 +7753,7 @@
         </is>
       </c>
       <c r="E319" t="n">
-        <v>21486</v>
+        <v>16</v>
       </c>
     </row>
     <row r="320">
@@ -7762,7 +7762,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -7776,7 +7776,7 @@
         </is>
       </c>
       <c r="E320" t="n">
-        <v>14673</v>
+        <v>32</v>
       </c>
     </row>
     <row r="321">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -7795,11 +7795,11 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E321" t="n">
-        <v>155811</v>
+        <v>40</v>
       </c>
     </row>
     <row r="322">
@@ -7808,21 +7808,21 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E322" t="n">
-        <v>39906</v>
+        <v>32</v>
       </c>
     </row>
     <row r="323">
@@ -7831,20 +7831,296 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
+          <t>1941 - EGE-SEPLAG</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Inativo</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>INATIVO CIVIL</t>
+        </is>
+      </c>
+      <c r="E323" t="n">
+        <v>1703</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>2161 - FUCAM</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>DIREÇÃO SUPERIOR</t>
+        </is>
+      </c>
+      <c r="E324" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>2161 - FUCAM</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
+        </is>
+      </c>
+      <c r="E325" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>2161 - FUCAM</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>TÉCNICA</t>
+        </is>
+      </c>
+      <c r="E326" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>2161 - FUCAM</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>2161 - FUCAM</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Inativo</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>INATIVO CIVIL</t>
+        </is>
+      </c>
+      <c r="E328" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
           <t>1261 - SEE</t>
         </is>
       </c>
-      <c r="C323" t="inlineStr">
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>DIREÇÃO SUPERIOR</t>
+        </is>
+      </c>
+      <c r="E329" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>4125</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>TÉCNICA</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>21486</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>ESPECIALIZADA</t>
+        </is>
+      </c>
+      <c r="E332" t="n">
+        <v>14673</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>DOCENTE</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>155811</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>39906</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
         <is>
           <t>Inativo</t>
         </is>
       </c>
-      <c r="D323" t="inlineStr">
+      <c r="D335" t="inlineStr">
         <is>
           <t>INATIVO CIVIL</t>
         </is>
       </c>
-      <c r="E323" t="n">
+      <c r="E335" t="n">
         <v>175450</v>
       </c>
     </row>

</xml_diff>